<commit_message>
Nuspalvoti Greitis lapo kintami stulpeliai ir eilutės
</commit_message>
<xml_diff>
--- a/PVZ1.xlsx
+++ b/PVZ1.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{2BCBD961-DBD3-4CBD-B361-331DD08C2361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Compatibility Report" sheetId="1" state="hidden" r:id="rId1"/>
@@ -1849,6 +1849,57 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1882,17 +1933,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1941,51 +1981,11 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="172" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2420,31 +2420,31 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="D2" s="266" t="s">
+      <c r="D2" s="269" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="267"/>
-      <c r="F2" s="267"/>
-      <c r="G2" s="267"/>
-      <c r="H2" s="267"/>
-      <c r="I2" s="267"/>
-      <c r="J2" s="267"/>
-      <c r="K2" s="267"/>
-      <c r="L2" s="267"/>
-      <c r="M2" s="267"/>
-      <c r="N2" s="267"/>
-      <c r="O2" s="267"/>
-      <c r="P2" s="267"/>
-      <c r="Q2" s="267"/>
-      <c r="R2" s="267"/>
-      <c r="S2" s="267"/>
-      <c r="T2" s="267"/>
-      <c r="U2" s="267"/>
-      <c r="V2" s="267"/>
-      <c r="W2" s="267"/>
-      <c r="X2" s="267"/>
-      <c r="Y2" s="267"/>
-      <c r="Z2" s="267"/>
+      <c r="E2" s="270"/>
+      <c r="F2" s="270"/>
+      <c r="G2" s="270"/>
+      <c r="H2" s="270"/>
+      <c r="I2" s="270"/>
+      <c r="J2" s="270"/>
+      <c r="K2" s="270"/>
+      <c r="L2" s="270"/>
+      <c r="M2" s="270"/>
+      <c r="N2" s="270"/>
+      <c r="O2" s="270"/>
+      <c r="P2" s="270"/>
+      <c r="Q2" s="270"/>
+      <c r="R2" s="270"/>
+      <c r="S2" s="270"/>
+      <c r="T2" s="270"/>
+      <c r="U2" s="270"/>
+      <c r="V2" s="270"/>
+      <c r="W2" s="270"/>
+      <c r="X2" s="270"/>
+      <c r="Y2" s="270"/>
+      <c r="Z2" s="270"/>
     </row>
     <row r="4" spans="1:28" s="10" customFormat="1" ht="126" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
@@ -2533,13 +2533,13 @@
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A5" s="261">
+      <c r="A5" s="277">
         <v>46063</v>
       </c>
-      <c r="B5" s="265">
+      <c r="B5" s="281">
         <v>5</v>
       </c>
-      <c r="C5" s="260" t="s">
+      <c r="C5" s="276" t="s">
         <v>29</v>
       </c>
       <c r="D5" s="85">
@@ -2630,14 +2630,14 @@
         <f>Aerodinamika!G27</f>
         <v>1.3179692000000001</v>
       </c>
-      <c r="AB5" s="259" t="s">
+      <c r="AB5" s="275" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A6" s="257"/>
-      <c r="B6" s="257"/>
-      <c r="C6" s="257"/>
+      <c r="A6" s="273"/>
+      <c r="B6" s="273"/>
+      <c r="C6" s="273"/>
       <c r="D6" s="85">
         <v>16</v>
       </c>
@@ -2722,12 +2722,12 @@
         <f>O5*X6</f>
         <v>0.79775867584824989</v>
       </c>
-      <c r="AB6" s="258"/>
+      <c r="AB6" s="274"/>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="257"/>
-      <c r="B7" s="257"/>
-      <c r="C7" s="257"/>
+      <c r="A7" s="273"/>
+      <c r="B7" s="273"/>
+      <c r="C7" s="273"/>
       <c r="D7" s="108">
         <v>31</v>
       </c>
@@ -2778,9 +2778,9 @@
       <c r="S7" s="58"/>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="257"/>
-      <c r="B8" s="257"/>
-      <c r="C8" s="257"/>
+      <c r="A8" s="273"/>
+      <c r="B8" s="273"/>
+      <c r="C8" s="273"/>
       <c r="D8" s="85">
         <v>60</v>
       </c>
@@ -2831,9 +2831,9 @@
       <c r="AA8" s="70"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A9" s="257"/>
-      <c r="B9" s="257"/>
-      <c r="C9" s="257"/>
+      <c r="A9" s="273"/>
+      <c r="B9" s="273"/>
+      <c r="C9" s="273"/>
       <c r="D9" s="85">
         <v>89</v>
       </c>
@@ -2877,9 +2877,9 @@
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A10" s="257"/>
-      <c r="B10" s="257"/>
-      <c r="C10" s="257"/>
+      <c r="A10" s="273"/>
+      <c r="B10" s="273"/>
+      <c r="C10" s="273"/>
       <c r="D10" s="85">
         <v>104</v>
       </c>
@@ -2923,9 +2923,9 @@
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A11" s="258"/>
-      <c r="B11" s="258"/>
-      <c r="C11" s="258"/>
+      <c r="A11" s="274"/>
+      <c r="B11" s="274"/>
+      <c r="C11" s="274"/>
       <c r="D11" s="85">
         <v>115</v>
       </c>
@@ -2994,18 +2994,18 @@
       <c r="D13" s="65" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="262" t="s">
+      <c r="E13" s="278" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="263"/>
-      <c r="G13" s="263"/>
-      <c r="H13" s="263"/>
-      <c r="I13" s="263"/>
-      <c r="J13" s="263"/>
-      <c r="K13" s="263"/>
-      <c r="L13" s="263"/>
-      <c r="M13" s="263"/>
-      <c r="N13" s="264"/>
+      <c r="F13" s="279"/>
+      <c r="G13" s="279"/>
+      <c r="H13" s="279"/>
+      <c r="I13" s="279"/>
+      <c r="J13" s="279"/>
+      <c r="K13" s="279"/>
+      <c r="L13" s="279"/>
+      <c r="M13" s="279"/>
+      <c r="N13" s="280"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" s="69"/>
@@ -3040,31 +3040,31 @@
       <c r="A17" s="69"/>
       <c r="B17" s="69"/>
       <c r="C17" s="69"/>
-      <c r="D17" s="268" t="s">
+      <c r="D17" s="271" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="267"/>
-      <c r="F17" s="267"/>
-      <c r="G17" s="267"/>
-      <c r="H17" s="267"/>
-      <c r="I17" s="267"/>
-      <c r="J17" s="267"/>
-      <c r="K17" s="267"/>
-      <c r="L17" s="267"/>
-      <c r="M17" s="267"/>
-      <c r="N17" s="267"/>
-      <c r="O17" s="267"/>
-      <c r="P17" s="267"/>
-      <c r="Q17" s="267"/>
-      <c r="R17" s="267"/>
-      <c r="S17" s="267"/>
-      <c r="T17" s="267"/>
-      <c r="U17" s="267"/>
-      <c r="V17" s="267"/>
-      <c r="W17" s="267"/>
-      <c r="X17" s="267"/>
-      <c r="Y17" s="267"/>
-      <c r="Z17" s="267"/>
+      <c r="E17" s="270"/>
+      <c r="F17" s="270"/>
+      <c r="G17" s="270"/>
+      <c r="H17" s="270"/>
+      <c r="I17" s="270"/>
+      <c r="J17" s="270"/>
+      <c r="K17" s="270"/>
+      <c r="L17" s="270"/>
+      <c r="M17" s="270"/>
+      <c r="N17" s="270"/>
+      <c r="O17" s="270"/>
+      <c r="P17" s="270"/>
+      <c r="Q17" s="270"/>
+      <c r="R17" s="270"/>
+      <c r="S17" s="270"/>
+      <c r="T17" s="270"/>
+      <c r="U17" s="270"/>
+      <c r="V17" s="270"/>
+      <c r="W17" s="270"/>
+      <c r="X17" s="270"/>
+      <c r="Y17" s="270"/>
+      <c r="Z17" s="270"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" s="69"/>
@@ -3170,9 +3170,9 @@
       </c>
     </row>
     <row r="20" spans="1:28" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="256"/>
-      <c r="B20" s="256"/>
-      <c r="C20" s="256"/>
+      <c r="A20" s="272"/>
+      <c r="B20" s="272"/>
+      <c r="C20" s="272"/>
       <c r="D20" s="59">
         <v>3</v>
       </c>
@@ -3249,12 +3249,12 @@
       <c r="AA20" s="59">
         <v>1.35</v>
       </c>
-      <c r="AB20" s="259"/>
+      <c r="AB20" s="275"/>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A21" s="257"/>
-      <c r="B21" s="257"/>
-      <c r="C21" s="257"/>
+      <c r="A21" s="273"/>
+      <c r="B21" s="273"/>
+      <c r="C21" s="273"/>
       <c r="D21" s="59">
         <v>15</v>
       </c>
@@ -3325,12 +3325,12 @@
         <f>O20*X21</f>
         <v>1.0671545706141217</v>
       </c>
-      <c r="AB21" s="258"/>
+      <c r="AB21" s="274"/>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A22" s="257"/>
-      <c r="B22" s="257"/>
-      <c r="C22" s="257"/>
+      <c r="A22" s="273"/>
+      <c r="B22" s="273"/>
+      <c r="C22" s="273"/>
       <c r="D22" s="65">
         <v>27</v>
       </c>
@@ -3369,9 +3369,9 @@
       <c r="S22" s="58"/>
     </row>
     <row r="23" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A23" s="257"/>
-      <c r="B23" s="257"/>
-      <c r="C23" s="257"/>
+      <c r="A23" s="273"/>
+      <c r="B23" s="273"/>
+      <c r="C23" s="273"/>
       <c r="D23" s="59">
         <v>4</v>
       </c>
@@ -3414,9 +3414,9 @@
       </c>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A24" s="257"/>
-      <c r="B24" s="257"/>
-      <c r="C24" s="257"/>
+      <c r="A24" s="273"/>
+      <c r="B24" s="273"/>
+      <c r="C24" s="273"/>
       <c r="D24" s="59">
         <v>5</v>
       </c>
@@ -3448,9 +3448,9 @@
       </c>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A25" s="257"/>
-      <c r="B25" s="257"/>
-      <c r="C25" s="257"/>
+      <c r="A25" s="273"/>
+      <c r="B25" s="273"/>
+      <c r="C25" s="273"/>
       <c r="D25" s="59">
         <v>6</v>
       </c>
@@ -3482,9 +3482,9 @@
       </c>
     </row>
     <row r="26" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A26" s="258"/>
-      <c r="B26" s="258"/>
-      <c r="C26" s="258"/>
+      <c r="A26" s="274"/>
+      <c r="B26" s="274"/>
+      <c r="C26" s="274"/>
       <c r="D26" s="59">
         <v>7</v>
       </c>
@@ -3518,17 +3518,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="YnNuFyjIZWP4o8siiNLOxJuXYMQvqdvZ9OrGGKpnMs1jyahS3pGpSVhE713S/7NZQvFDz0ZfCGMwTjhjC08CdQ==" saltValue="gCAgvRWICbIOkCsyhMCWFQ==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="11">
-    <mergeCell ref="D2:Z2"/>
-    <mergeCell ref="D17:Z17"/>
-    <mergeCell ref="B20:B26"/>
-    <mergeCell ref="C20:C26"/>
-    <mergeCell ref="A20:A26"/>
     <mergeCell ref="AB5:AB6"/>
     <mergeCell ref="AB20:AB21"/>
     <mergeCell ref="C5:C11"/>
     <mergeCell ref="A5:A11"/>
     <mergeCell ref="E13:N13"/>
     <mergeCell ref="B5:B11"/>
+    <mergeCell ref="D2:Z2"/>
+    <mergeCell ref="D17:Z17"/>
+    <mergeCell ref="B20:B26"/>
+    <mergeCell ref="C20:C26"/>
+    <mergeCell ref="A20:A26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3575,18 +3575,18 @@
       <c r="I2" s="10"/>
     </row>
     <row r="3" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="273" t="s">
+      <c r="A3" s="286" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="267"/>
-      <c r="C3" s="267"/>
-      <c r="D3" s="267"/>
-      <c r="E3" s="267"/>
-      <c r="F3" s="267"/>
-      <c r="G3" s="267"/>
-      <c r="H3" s="267"/>
-      <c r="I3" s="267"/>
-      <c r="J3" s="267"/>
+      <c r="B3" s="270"/>
+      <c r="C3" s="270"/>
+      <c r="D3" s="270"/>
+      <c r="E3" s="270"/>
+      <c r="F3" s="270"/>
+      <c r="G3" s="270"/>
+      <c r="H3" s="270"/>
+      <c r="I3" s="270"/>
+      <c r="J3" s="270"/>
     </row>
     <row r="4" spans="1:12" ht="14" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
@@ -3733,46 +3733,46 @@
       <c r="L10" s="27"/>
     </row>
     <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H11" s="270" t="s">
+      <c r="H11" s="283" t="s">
         <v>55</v>
       </c>
-      <c r="I11" s="269" t="s">
+      <c r="I11" s="282" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H12" s="271"/>
-      <c r="I12" s="257"/>
+      <c r="H12" s="284"/>
+      <c r="I12" s="273"/>
     </row>
     <row r="13" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H13" s="271"/>
-      <c r="I13" s="257"/>
+      <c r="H13" s="284"/>
+      <c r="I13" s="273"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H14" s="271"/>
-      <c r="I14" s="257"/>
+      <c r="H14" s="284"/>
+      <c r="I14" s="273"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H15" s="271"/>
-      <c r="I15" s="257"/>
+      <c r="H15" s="284"/>
+      <c r="I15" s="273"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H16" s="271"/>
-      <c r="I16" s="257"/>
+      <c r="H16" s="284"/>
+      <c r="I16" s="273"/>
     </row>
     <row r="17" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H17" s="271"/>
-      <c r="I17" s="257"/>
+      <c r="H17" s="284"/>
+      <c r="I17" s="273"/>
     </row>
     <row r="18" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H18" s="272"/>
-      <c r="I18" s="257"/>
+      <c r="H18" s="285"/>
+      <c r="I18" s="273"/>
     </row>
     <row r="19" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I19" s="257"/>
+      <c r="I19" s="273"/>
     </row>
     <row r="20" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I20" s="258"/>
+      <c r="I20" s="274"/>
     </row>
     <row r="21" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I21" s="32"/>
@@ -3835,35 +3835,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="277" t="s">
+      <c r="C1" s="290" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="267"/>
+      <c r="D1" s="270"/>
       <c r="E1" s="15"/>
       <c r="S1" s="16"/>
     </row>
     <row r="2" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="282" t="s">
+      <c r="A2" s="295" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="267"/>
-      <c r="C2" s="267"/>
-      <c r="D2" s="267"/>
-      <c r="E2" s="267"/>
-      <c r="F2" s="267"/>
-      <c r="G2" s="267"/>
-      <c r="H2" s="267"/>
-      <c r="I2" s="267"/>
-      <c r="J2" s="267"/>
-      <c r="K2" s="267"/>
-      <c r="L2" s="267"/>
-      <c r="M2" s="267"/>
-      <c r="N2" s="267"/>
-      <c r="O2" s="267"/>
-      <c r="P2" s="267"/>
-      <c r="Q2" s="267"/>
-      <c r="R2" s="267"/>
-      <c r="S2" s="267"/>
+      <c r="B2" s="270"/>
+      <c r="C2" s="270"/>
+      <c r="D2" s="270"/>
+      <c r="E2" s="270"/>
+      <c r="F2" s="270"/>
+      <c r="G2" s="270"/>
+      <c r="H2" s="270"/>
+      <c r="I2" s="270"/>
+      <c r="J2" s="270"/>
+      <c r="K2" s="270"/>
+      <c r="L2" s="270"/>
+      <c r="M2" s="270"/>
+      <c r="N2" s="270"/>
+      <c r="O2" s="270"/>
+      <c r="P2" s="270"/>
+      <c r="Q2" s="270"/>
+      <c r="R2" s="270"/>
+      <c r="S2" s="270"/>
     </row>
     <row r="3" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
@@ -3965,7 +3965,7 @@
       <c r="B6" s="130" t="s">
         <v>77</v>
       </c>
-      <c r="C6" s="278" t="str">
+      <c r="C6" s="291" t="str">
         <f>Greitis!C5</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -4037,7 +4037,7 @@
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="144"/>
       <c r="B7" s="145"/>
-      <c r="C7" s="279"/>
+      <c r="C7" s="292"/>
       <c r="D7" s="147"/>
       <c r="E7" s="148"/>
       <c r="F7" s="133">
@@ -4100,7 +4100,7 @@
     <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="144"/>
       <c r="B8" s="145"/>
-      <c r="C8" s="279"/>
+      <c r="C8" s="292"/>
       <c r="D8" s="147"/>
       <c r="E8" s="148"/>
       <c r="F8" s="133">
@@ -4163,7 +4163,7 @@
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="146"/>
       <c r="B9" s="146"/>
-      <c r="C9" s="279"/>
+      <c r="C9" s="292"/>
       <c r="D9" s="153"/>
       <c r="E9" s="153"/>
       <c r="F9" s="133">
@@ -4229,7 +4229,7 @@
     <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="146"/>
       <c r="B10" s="146"/>
-      <c r="C10" s="279"/>
+      <c r="C10" s="292"/>
       <c r="D10" s="153"/>
       <c r="E10" s="153"/>
       <c r="F10" s="133">
@@ -4279,20 +4279,20 @@
       </c>
       <c r="R10" s="153"/>
       <c r="S10" s="153"/>
-      <c r="T10" s="274" t="s">
+      <c r="T10" s="287" t="s">
         <v>80</v>
       </c>
-      <c r="U10" s="274" t="s">
+      <c r="U10" s="287" t="s">
         <v>81</v>
       </c>
-      <c r="V10" s="281" t="s">
+      <c r="V10" s="294" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" s="146"/>
       <c r="B11" s="146"/>
-      <c r="C11" s="279"/>
+      <c r="C11" s="292"/>
       <c r="D11" s="153"/>
       <c r="E11" s="153"/>
       <c r="F11" s="133">
@@ -4342,14 +4342,14 @@
       </c>
       <c r="R11" s="153"/>
       <c r="S11" s="153"/>
-      <c r="T11" s="275"/>
-      <c r="U11" s="275"/>
-      <c r="V11" s="275"/>
+      <c r="T11" s="288"/>
+      <c r="U11" s="288"/>
+      <c r="V11" s="288"/>
     </row>
     <row r="12" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="154"/>
       <c r="B12" s="154"/>
-      <c r="C12" s="280"/>
+      <c r="C12" s="293"/>
       <c r="D12" s="155"/>
       <c r="E12" s="155"/>
       <c r="F12" s="133">
@@ -4399,9 +4399,9 @@
       </c>
       <c r="R12" s="155"/>
       <c r="S12" s="155"/>
-      <c r="T12" s="276"/>
-      <c r="U12" s="276"/>
-      <c r="V12" s="276"/>
+      <c r="T12" s="289"/>
+      <c r="U12" s="289"/>
+      <c r="V12" s="289"/>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="L13" s="156">
@@ -4442,7 +4442,7 @@
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="C17" s="278" t="str">
+      <c r="C17" s="291" t="str">
         <f t="shared" si="1"/>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -4513,7 +4513,7 @@
     <row r="18" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A18" s="163"/>
       <c r="B18" s="164"/>
-      <c r="C18" s="279"/>
+      <c r="C18" s="292"/>
       <c r="D18" s="147"/>
       <c r="E18" s="148"/>
       <c r="F18" s="133">
@@ -4570,7 +4570,7 @@
     <row r="19" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A19" s="163"/>
       <c r="B19" s="164"/>
-      <c r="C19" s="279"/>
+      <c r="C19" s="292"/>
       <c r="D19" s="147"/>
       <c r="E19" s="148"/>
       <c r="F19" s="133">
@@ -4627,7 +4627,7 @@
     <row r="20" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A20" s="153"/>
       <c r="B20" s="153"/>
-      <c r="C20" s="279"/>
+      <c r="C20" s="292"/>
       <c r="D20" s="153"/>
       <c r="E20" s="153"/>
       <c r="F20" s="133">
@@ -4684,7 +4684,7 @@
     <row r="21" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A21" s="153"/>
       <c r="B21" s="153"/>
-      <c r="C21" s="279"/>
+      <c r="C21" s="292"/>
       <c r="D21" s="153"/>
       <c r="E21" s="153"/>
       <c r="F21" s="133">
@@ -4741,7 +4741,7 @@
     <row r="22" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A22" s="153"/>
       <c r="B22" s="153"/>
-      <c r="C22" s="279"/>
+      <c r="C22" s="292"/>
       <c r="D22" s="153"/>
       <c r="E22" s="153"/>
       <c r="F22" s="133">
@@ -4798,7 +4798,7 @@
     <row r="23" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A23" s="155"/>
       <c r="B23" s="155"/>
-      <c r="C23" s="280"/>
+      <c r="C23" s="293"/>
       <c r="D23" s="155"/>
       <c r="E23" s="155"/>
       <c r="F23" s="133">
@@ -4972,10 +4972,10 @@
     <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="166"/>
       <c r="B1" s="166"/>
-      <c r="C1" s="283" t="s">
+      <c r="C1" s="256" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="284"/>
+      <c r="D1" s="257"/>
       <c r="E1" s="166"/>
       <c r="F1" s="166"/>
       <c r="G1" s="166"/>
@@ -4991,19 +4991,19 @@
     <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="166"/>
       <c r="B2" s="166"/>
-      <c r="C2" s="287" t="s">
+      <c r="C2" s="267" t="s">
         <v>91</v>
       </c>
-      <c r="D2" s="284"/>
-      <c r="E2" s="284"/>
-      <c r="F2" s="284"/>
-      <c r="G2" s="284"/>
-      <c r="H2" s="284"/>
-      <c r="I2" s="284"/>
-      <c r="J2" s="284"/>
-      <c r="K2" s="284"/>
-      <c r="L2" s="284"/>
-      <c r="M2" s="284"/>
+      <c r="D2" s="257"/>
+      <c r="E2" s="257"/>
+      <c r="F2" s="257"/>
+      <c r="G2" s="257"/>
+      <c r="H2" s="257"/>
+      <c r="I2" s="257"/>
+      <c r="J2" s="257"/>
+      <c r="K2" s="257"/>
+      <c r="L2" s="257"/>
+      <c r="M2" s="257"/>
       <c r="N2" s="166"/>
       <c r="Q2" s="16"/>
     </row>
@@ -5093,7 +5093,7 @@
         <f>Paėmimas!B6</f>
         <v>3</v>
       </c>
-      <c r="C6" s="285" t="str">
+      <c r="C6" s="296" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -5145,7 +5145,7 @@
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="180"/>
       <c r="B7" s="181"/>
-      <c r="C7" s="286"/>
+      <c r="C7" s="262"/>
       <c r="D7" s="127">
         <f>Paėmimas!L7</f>
         <v>3.5999999999999997E-2</v>
@@ -5182,7 +5182,7 @@
     <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="180"/>
       <c r="B8" s="181"/>
-      <c r="C8" s="286"/>
+      <c r="C8" s="262"/>
       <c r="D8" s="127">
         <f>Paėmimas!L8</f>
         <v>3.5999999999999997E-2</v>
@@ -5219,7 +5219,7 @@
     <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="180"/>
       <c r="B9" s="181"/>
-      <c r="C9" s="286"/>
+      <c r="C9" s="262"/>
       <c r="D9" s="127">
         <f>Paėmimas!L9</f>
         <v>3.5999999999999997E-2</v>
@@ -5256,7 +5256,7 @@
     <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="180"/>
       <c r="B10" s="181"/>
-      <c r="C10" s="286"/>
+      <c r="C10" s="262"/>
       <c r="D10" s="127">
         <f>Paėmimas!L10</f>
         <v>3.5999999999999997E-2</v>
@@ -5293,7 +5293,7 @@
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="180"/>
       <c r="B11" s="181"/>
-      <c r="C11" s="286"/>
+      <c r="C11" s="262"/>
       <c r="D11" s="127">
         <f>Paėmimas!L11</f>
         <v>3.3000000000000002E-2</v>
@@ -5330,7 +5330,7 @@
     <row r="12" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="185"/>
       <c r="B12" s="186"/>
-      <c r="C12" s="286"/>
+      <c r="C12" s="262"/>
       <c r="D12" s="127">
         <f>Paėmimas!L12</f>
         <v>0.03</v>
@@ -5447,7 +5447,7 @@
         <f>Paėmimas!B17</f>
         <v>3</v>
       </c>
-      <c r="C17" s="285" t="str">
+      <c r="C17" s="296" t="str">
         <f>Paėmimas!C17</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -5499,7 +5499,7 @@
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="180"/>
       <c r="B18" s="181"/>
-      <c r="C18" s="286"/>
+      <c r="C18" s="262"/>
       <c r="D18" s="127">
         <f>Paėmimas!L18</f>
         <v>3.3000000000000002E-2</v>
@@ -5536,7 +5536,7 @@
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="180"/>
       <c r="B19" s="181"/>
-      <c r="C19" s="286"/>
+      <c r="C19" s="262"/>
       <c r="D19" s="127">
         <f>Paėmimas!L19</f>
         <v>3.3000000000000002E-2</v>
@@ -5573,7 +5573,7 @@
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="180"/>
       <c r="B20" s="181"/>
-      <c r="C20" s="286"/>
+      <c r="C20" s="262"/>
       <c r="D20" s="127">
         <f>Paėmimas!L20</f>
         <v>3.5999999999999997E-2</v>
@@ -5610,7 +5610,7 @@
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="180"/>
       <c r="B21" s="181"/>
-      <c r="C21" s="286"/>
+      <c r="C21" s="262"/>
       <c r="D21" s="127">
         <f>Paėmimas!L21</f>
         <v>3.3000000000000002E-2</v>
@@ -5647,7 +5647,7 @@
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="180"/>
       <c r="B22" s="181"/>
-      <c r="C22" s="286"/>
+      <c r="C22" s="262"/>
       <c r="D22" s="127">
         <f>Paėmimas!L22</f>
         <v>3.3000000000000002E-2</v>
@@ -5684,7 +5684,7 @@
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="185"/>
       <c r="B23" s="186"/>
-      <c r="C23" s="286"/>
+      <c r="C23" s="262"/>
       <c r="D23" s="127">
         <f>Paėmimas!L23</f>
         <v>3.3000000000000002E-2</v>
@@ -9581,10 +9581,10 @@
     <row r="1" spans="1:28" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="166"/>
       <c r="B1" s="166"/>
-      <c r="C1" s="283" t="s">
+      <c r="C1" s="256" t="s">
         <v>109</v>
       </c>
-      <c r="D1" s="284"/>
+      <c r="D1" s="257"/>
       <c r="E1" s="166"/>
       <c r="F1" s="166"/>
       <c r="G1" s="166"/>
@@ -9611,22 +9611,22 @@
       <c r="AB1" s="166"/>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A2" s="287" t="s">
+      <c r="A2" s="267" t="s">
         <v>110</v>
       </c>
-      <c r="B2" s="284"/>
-      <c r="C2" s="284"/>
-      <c r="D2" s="284"/>
-      <c r="E2" s="284"/>
-      <c r="F2" s="284"/>
-      <c r="G2" s="284"/>
-      <c r="H2" s="284"/>
-      <c r="I2" s="284"/>
-      <c r="J2" s="284"/>
-      <c r="K2" s="284"/>
-      <c r="L2" s="284"/>
-      <c r="M2" s="284"/>
-      <c r="N2" s="284"/>
+      <c r="B2" s="257"/>
+      <c r="C2" s="257"/>
+      <c r="D2" s="257"/>
+      <c r="E2" s="257"/>
+      <c r="F2" s="257"/>
+      <c r="G2" s="257"/>
+      <c r="H2" s="257"/>
+      <c r="I2" s="257"/>
+      <c r="J2" s="257"/>
+      <c r="K2" s="257"/>
+      <c r="L2" s="257"/>
+      <c r="M2" s="257"/>
+      <c r="N2" s="257"/>
       <c r="O2" s="169"/>
       <c r="P2" s="166"/>
       <c r="Q2" s="166"/>
@@ -9773,7 +9773,7 @@
         <f>Svėrimas!A6</f>
         <v>3</v>
       </c>
-      <c r="C6" s="288" t="str">
+      <c r="C6" s="297" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -9844,7 +9844,7 @@
     <row r="7" spans="1:28" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="200"/>
       <c r="B7" s="201"/>
-      <c r="C7" s="286"/>
+      <c r="C7" s="262"/>
       <c r="D7" s="212"/>
       <c r="E7" s="203"/>
       <c r="F7" s="213"/>
@@ -9874,7 +9874,7 @@
     <row r="8" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="217"/>
       <c r="B8" s="211"/>
-      <c r="C8" s="289"/>
+      <c r="C8" s="263"/>
       <c r="D8" s="212"/>
       <c r="E8" s="203"/>
       <c r="F8" s="213"/>
@@ -9944,12 +9944,12 @@
     <row r="1" spans="1:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="166"/>
       <c r="B1" s="166"/>
-      <c r="C1" s="283" t="s">
+      <c r="C1" s="256" t="s">
         <v>122</v>
       </c>
-      <c r="D1" s="284"/>
-      <c r="E1" s="284"/>
-      <c r="F1" s="284"/>
+      <c r="D1" s="257"/>
+      <c r="E1" s="257"/>
+      <c r="F1" s="257"/>
       <c r="G1" s="166"/>
       <c r="H1" s="166"/>
       <c r="I1" s="166"/>
@@ -9961,23 +9961,23 @@
       <c r="O1" s="166"/>
     </row>
     <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="287" t="s">
+      <c r="A2" s="267" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="284"/>
-      <c r="C2" s="284"/>
-      <c r="D2" s="284"/>
-      <c r="E2" s="284"/>
-      <c r="F2" s="284"/>
-      <c r="G2" s="284"/>
-      <c r="H2" s="284"/>
-      <c r="I2" s="284"/>
-      <c r="J2" s="284"/>
-      <c r="K2" s="284"/>
-      <c r="L2" s="284"/>
-      <c r="M2" s="284"/>
-      <c r="N2" s="284"/>
-      <c r="O2" s="284"/>
+      <c r="B2" s="257"/>
+      <c r="C2" s="257"/>
+      <c r="D2" s="257"/>
+      <c r="E2" s="257"/>
+      <c r="F2" s="257"/>
+      <c r="G2" s="257"/>
+      <c r="H2" s="257"/>
+      <c r="I2" s="257"/>
+      <c r="J2" s="257"/>
+      <c r="K2" s="257"/>
+      <c r="L2" s="257"/>
+      <c r="M2" s="257"/>
+      <c r="N2" s="257"/>
+      <c r="O2" s="257"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="166"/>
@@ -9997,49 +9997,49 @@
       <c r="O3" s="166"/>
     </row>
     <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="295" t="s">
+      <c r="A4" s="265" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="295" t="s">
+      <c r="B4" s="265" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="290" t="s">
+      <c r="C4" s="258" t="s">
         <v>124</v>
       </c>
-      <c r="D4" s="290" t="s">
+      <c r="D4" s="258" t="s">
         <v>125</v>
       </c>
-      <c r="E4" s="290" t="s">
+      <c r="E4" s="258" t="s">
         <v>126</v>
       </c>
-      <c r="F4" s="291"/>
-      <c r="G4" s="292"/>
-      <c r="H4" s="290" t="s">
+      <c r="F4" s="259"/>
+      <c r="G4" s="260"/>
+      <c r="H4" s="258" t="s">
         <v>127</v>
       </c>
-      <c r="I4" s="290" t="s">
+      <c r="I4" s="258" t="s">
         <v>128</v>
       </c>
-      <c r="J4" s="290" t="s">
+      <c r="J4" s="258" t="s">
         <v>129</v>
       </c>
-      <c r="K4" s="291"/>
-      <c r="L4" s="292"/>
-      <c r="M4" s="290" t="s">
+      <c r="K4" s="259"/>
+      <c r="L4" s="260"/>
+      <c r="M4" s="258" t="s">
         <v>130</v>
       </c>
-      <c r="N4" s="290" t="s">
+      <c r="N4" s="258" t="s">
         <v>127</v>
       </c>
-      <c r="O4" s="297" t="s">
+      <c r="O4" s="268" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="296"/>
-      <c r="B5" s="296"/>
-      <c r="C5" s="294"/>
-      <c r="D5" s="294"/>
+      <c r="A5" s="266"/>
+      <c r="B5" s="266"/>
+      <c r="C5" s="264"/>
+      <c r="D5" s="264"/>
       <c r="E5" s="118">
         <v>1</v>
       </c>
@@ -10049,8 +10049,8 @@
       <c r="G5" s="118">
         <v>3</v>
       </c>
-      <c r="H5" s="294"/>
-      <c r="I5" s="294"/>
+      <c r="H5" s="264"/>
+      <c r="I5" s="264"/>
       <c r="J5" s="118">
         <v>1</v>
       </c>
@@ -10060,16 +10060,16 @@
       <c r="L5" s="118">
         <v>3</v>
       </c>
-      <c r="M5" s="294"/>
-      <c r="N5" s="294"/>
-      <c r="O5" s="294"/>
+      <c r="M5" s="264"/>
+      <c r="N5" s="264"/>
+      <c r="O5" s="264"/>
     </row>
     <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="224" t="str">
         <f>Paėmimas!B6</f>
         <v>3</v>
       </c>
-      <c r="B6" s="293" t="str">
+      <c r="B6" s="261" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -10118,7 +10118,7 @@
     </row>
     <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="184"/>
-      <c r="B7" s="286"/>
+      <c r="B7" s="262"/>
       <c r="C7" s="232"/>
       <c r="D7" s="229"/>
       <c r="E7" s="233"/>
@@ -10138,7 +10138,7 @@
     </row>
     <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="184"/>
-      <c r="B8" s="286"/>
+      <c r="B8" s="262"/>
       <c r="C8" s="232"/>
       <c r="D8" s="237"/>
       <c r="E8" s="233"/>
@@ -10158,7 +10158,7 @@
     </row>
     <row r="9" spans="1:16" ht="17" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="184"/>
-      <c r="B9" s="286"/>
+      <c r="B9" s="262"/>
       <c r="C9" s="232">
         <v>2</v>
       </c>
@@ -10195,7 +10195,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="184"/>
-      <c r="B10" s="286"/>
+      <c r="B10" s="262"/>
       <c r="C10" s="232"/>
       <c r="D10" s="237"/>
       <c r="E10" s="233"/>
@@ -10212,7 +10212,7 @@
     </row>
     <row r="11" spans="1:16" ht="17" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="184"/>
-      <c r="B11" s="286"/>
+      <c r="B11" s="262"/>
       <c r="C11" s="232">
         <v>41</v>
       </c>
@@ -10248,7 +10248,7 @@
     </row>
     <row r="12" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="184"/>
-      <c r="B12" s="286"/>
+      <c r="B12" s="262"/>
       <c r="C12" s="245" t="s">
         <v>135</v>
       </c>
@@ -10284,7 +10284,7 @@
     </row>
     <row r="13" spans="1:16" ht="17" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="184"/>
-      <c r="B13" s="286"/>
+      <c r="B13" s="262"/>
       <c r="C13" s="249" t="s">
         <v>137</v>
       </c>
@@ -10320,7 +10320,7 @@
     </row>
     <row r="14" spans="1:16" ht="17" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="184"/>
-      <c r="B14" s="286"/>
+      <c r="B14" s="262"/>
       <c r="C14" s="249" t="s">
         <v>139</v>
       </c>
@@ -10356,7 +10356,7 @@
     </row>
     <row r="15" spans="1:16" ht="17" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="184"/>
-      <c r="B15" s="286"/>
+      <c r="B15" s="262"/>
       <c r="C15" s="250" t="s">
         <v>141</v>
       </c>
@@ -10392,7 +10392,7 @@
     </row>
     <row r="16" spans="1:16" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="189"/>
-      <c r="B16" s="289"/>
+      <c r="B16" s="263"/>
       <c r="C16" s="232"/>
       <c r="D16" s="251"/>
       <c r="E16" s="173"/>
@@ -10497,9 +10497,9 @@
       <c r="A3" s="298" t="s">
         <v>144</v>
       </c>
-      <c r="B3" s="267"/>
-      <c r="C3" s="267"/>
-      <c r="D3" s="267"/>
+      <c r="B3" s="270"/>
+      <c r="C3" s="270"/>
+      <c r="D3" s="270"/>
     </row>
     <row r="5" spans="1:4" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="48" t="s">
@@ -10543,6 +10543,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentas" ma:contentTypeID="0x010100BAB57CF81AE55C4698AAD22D302297F0" ma:contentTypeVersion="18" ma:contentTypeDescription="Kurkite naują dokumentą." ma:contentTypeScope="" ma:versionID="49ab401eb4052690d2a2629974c22fd6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="453e7e53-5eb2-45cf-b2ab-34c867e554b8" xmlns:ns3="aa0d983d-359a-438c-9953-3af1a8ac0831" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ab9969d50e0b13c63bc5bd0499c928dc" ns2:_="" ns3:_="">
     <xsd:import namespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
@@ -10797,27 +10817,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AA6EE5C-752B-4FD7-A005-65DDA547B7D6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BBA06BC-36D1-4FA0-837A-73611C8B64E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FBF118E-AD3B-46FF-9D16-3F282B2B316B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10834,23 +10853,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BBA06BC-36D1-4FA0-837A-73611C8B64E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AA6EE5C-752B-4FD7-A005-65DDA547B7D6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
-    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Pakeistas A, B, C stulpelių lygiavimas ir suliejimas
</commit_message>
<xml_diff>
--- a/PVZ1.xlsx
+++ b/PVZ1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="Šios_darbaknygės" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agentura2020.sharepoint.com/sites/VidurioLietuvosaplinkostyrimuskyrius/Bendrai naudojami dokumentai/EB7-16 Metodų bylos/EB-114 Metodo byla SVPATD3-3 KD/Skaičiuoklės/Įteisinimo pvz/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agentura2020.sharepoint.com/sites/VidurioLietuvosaplinkostyrimuskyrius/Bendrai naudojami dokumentai/EB7-014 Darbuotojų failai/Tomo/Python 3.14.3/Skaiciavimai/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="155" documentId="8_{6218F508-2438-4EC7-8B4D-5D6F3C7CDB90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{201A47C8-B92F-45CF-9C07-2B82262E0461}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="821" firstSheet="1" activeTab="1" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="6" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Compatibility Report" sheetId="4" state="hidden" r:id="rId1"/>
@@ -2694,6 +2694,30 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="29" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
@@ -2730,30 +2754,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="29" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -2817,6 +2817,23 @@
     <xf numFmtId="169" fontId="4" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -2851,23 +2868,6 @@
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -3183,16 +3183,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ABD58BE-2006-42BB-8F0B-A2F613982E7B}">
   <sheetPr codeName="Lapas1"/>
   <dimension ref="B1:E10"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.140625" customWidth="1"/>
-    <col min="2" max="2" width="64.42578125" customWidth="1"/>
-    <col min="3" max="3" width="1.5703125" customWidth="1"/>
-    <col min="4" max="4" width="5.5703125" customWidth="1"/>
+    <col min="1" max="1" width="1.1796875" customWidth="1"/>
+    <col min="2" max="2" width="64.453125" customWidth="1"/>
+    <col min="3" max="3" width="1.54296875" customWidth="1"/>
+    <col min="4" max="4" width="5.54296875" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:5" ht="13" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3200,7 +3200,7 @@
       <c r="D1" s="5"/>
       <c r="E1" s="5"/>
     </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:5" ht="13" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
@@ -3208,13 +3208,13 @@
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
     </row>
-    <row r="4" spans="2:5" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:5" ht="37.5" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
@@ -3222,13 +3222,13 @@
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:5" ht="13" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
@@ -3238,13 +3238,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="2:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
     </row>
-    <row r="8" spans="2:5" ht="39" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>5</v>
       </c>
@@ -3254,13 +3254,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="6"/>
@@ -3275,61 +3275,61 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B3F6816-A3F5-4347-BE94-F213DC59E543}">
   <dimension ref="A3:AB31"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" style="131" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" style="131" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" style="131" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" style="131" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" style="131" customWidth="1"/>
-    <col min="6" max="6" width="11.28515625" style="131" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" style="131" customWidth="1"/>
-    <col min="8" max="12" width="9.140625" style="131"/>
-    <col min="13" max="13" width="11.140625" style="131" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" style="131" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" style="131"/>
-    <col min="16" max="16" width="10.5703125" style="131" customWidth="1"/>
-    <col min="17" max="17" width="9.5703125" style="131" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.140625" style="131"/>
-    <col min="19" max="19" width="11.28515625" style="131" customWidth="1"/>
-    <col min="20" max="20" width="11.7109375" style="131" customWidth="1"/>
+    <col min="1" max="1" width="11.26953125" style="131" customWidth="1"/>
+    <col min="2" max="2" width="11.1796875" style="131" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" style="131" customWidth="1"/>
+    <col min="4" max="4" width="10.26953125" style="131" customWidth="1"/>
+    <col min="5" max="5" width="11.1796875" style="131" customWidth="1"/>
+    <col min="6" max="6" width="11.26953125" style="131" customWidth="1"/>
+    <col min="7" max="7" width="10.54296875" style="131" customWidth="1"/>
+    <col min="8" max="12" width="9.1796875" style="131"/>
+    <col min="13" max="13" width="11.1796875" style="131" customWidth="1"/>
+    <col min="14" max="14" width="11.453125" style="131" customWidth="1"/>
+    <col min="15" max="15" width="9.1796875" style="131"/>
+    <col min="16" max="16" width="10.54296875" style="131" customWidth="1"/>
+    <col min="17" max="17" width="9.54296875" style="131" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.1796875" style="131"/>
+    <col min="19" max="19" width="11.26953125" style="131" customWidth="1"/>
+    <col min="20" max="20" width="11.7265625" style="131" customWidth="1"/>
     <col min="21" max="21" width="10" style="131" customWidth="1"/>
-    <col min="22" max="22" width="11.7109375" style="131" customWidth="1"/>
-    <col min="23" max="23" width="11.42578125" style="131" customWidth="1"/>
-    <col min="24" max="24" width="10.28515625" style="131" customWidth="1"/>
-    <col min="25" max="25" width="9.5703125" style="131" customWidth="1"/>
-    <col min="26" max="26" width="9.85546875" style="131" customWidth="1"/>
-    <col min="27" max="16384" width="9.140625" style="131"/>
+    <col min="22" max="22" width="11.7265625" style="131" customWidth="1"/>
+    <col min="23" max="23" width="11.453125" style="131" customWidth="1"/>
+    <col min="24" max="24" width="10.26953125" style="131" customWidth="1"/>
+    <col min="25" max="25" width="9.54296875" style="131" customWidth="1"/>
+    <col min="26" max="26" width="9.81640625" style="131" customWidth="1"/>
+    <col min="27" max="16384" width="9.1796875" style="131"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="D3" s="262" t="s">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="D3" s="268" t="s">
         <v>109</v>
       </c>
-      <c r="E3" s="262"/>
-      <c r="F3" s="262"/>
-      <c r="G3" s="262"/>
-      <c r="H3" s="262"/>
-      <c r="I3" s="262"/>
-      <c r="J3" s="262"/>
-      <c r="K3" s="262"/>
-      <c r="L3" s="262"/>
-      <c r="M3" s="262"/>
-      <c r="N3" s="262"/>
-      <c r="O3" s="262"/>
-      <c r="P3" s="262"/>
-      <c r="Q3" s="262"/>
-      <c r="R3" s="262"/>
-      <c r="S3" s="262"/>
-      <c r="T3" s="262"/>
-      <c r="U3" s="262"/>
-      <c r="V3" s="262"/>
-      <c r="W3" s="262"/>
-      <c r="X3" s="262"/>
-      <c r="Y3" s="262"/>
-      <c r="Z3" s="262"/>
-    </row>
-    <row r="5" spans="1:28" s="10" customFormat="1" ht="150" x14ac:dyDescent="0.2">
+      <c r="E3" s="268"/>
+      <c r="F3" s="268"/>
+      <c r="G3" s="268"/>
+      <c r="H3" s="268"/>
+      <c r="I3" s="268"/>
+      <c r="J3" s="268"/>
+      <c r="K3" s="268"/>
+      <c r="L3" s="268"/>
+      <c r="M3" s="268"/>
+      <c r="N3" s="268"/>
+      <c r="O3" s="268"/>
+      <c r="P3" s="268"/>
+      <c r="Q3" s="268"/>
+      <c r="R3" s="268"/>
+      <c r="S3" s="268"/>
+      <c r="T3" s="268"/>
+      <c r="U3" s="268"/>
+      <c r="V3" s="268"/>
+      <c r="W3" s="268"/>
+      <c r="X3" s="268"/>
+      <c r="Y3" s="268"/>
+      <c r="Z3" s="268"/>
+    </row>
+    <row r="5" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>8</v>
       </c>
@@ -3415,14 +3415,14 @@
         <v>129</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="272" t="s">
+    <row r="6" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="263" t="s">
         <v>148</v>
       </c>
-      <c r="B6" s="263" t="s">
+      <c r="B6" s="269" t="s">
         <v>147</v>
       </c>
-      <c r="C6" s="264" t="s">
+      <c r="C6" s="270" t="s">
         <v>149</v>
       </c>
       <c r="D6" s="135">
@@ -3513,14 +3513,14 @@
         <f>Aerodinamika!G31</f>
         <v>1.2973599999999996</v>
       </c>
-      <c r="AB6" s="260" t="s">
+      <c r="AB6" s="266" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A7" s="273"/>
-      <c r="B7" s="263"/>
-      <c r="C7" s="264"/>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A7" s="264"/>
+      <c r="B7" s="269"/>
+      <c r="C7" s="270"/>
       <c r="D7" s="135">
         <v>39</v>
       </c>
@@ -3605,12 +3605,12 @@
         <f>O6*X7</f>
         <v>0.34740732161375365</v>
       </c>
-      <c r="AB7" s="261"/>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A8" s="273"/>
-      <c r="B8" s="263"/>
-      <c r="C8" s="264"/>
+      <c r="AB7" s="267"/>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A8" s="264"/>
+      <c r="B8" s="269"/>
+      <c r="C8" s="270"/>
       <c r="D8" s="152">
         <v>71</v>
       </c>
@@ -3660,10 +3660,10 @@
       <c r="R8" s="157"/>
       <c r="S8" s="157"/>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A9" s="273"/>
-      <c r="B9" s="263"/>
-      <c r="C9" s="264"/>
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A9" s="264"/>
+      <c r="B9" s="269"/>
+      <c r="C9" s="270"/>
       <c r="D9" s="135">
         <v>116</v>
       </c>
@@ -3717,10 +3717,10 @@
         <v>130</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A10" s="273"/>
-      <c r="B10" s="263"/>
-      <c r="C10" s="264"/>
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A10" s="264"/>
+      <c r="B10" s="269"/>
+      <c r="C10" s="270"/>
       <c r="D10" s="135">
         <v>200</v>
       </c>
@@ -3763,10 +3763,10 @@
         <v>4.1856303808885986</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A11" s="273"/>
-      <c r="B11" s="263"/>
-      <c r="C11" s="264"/>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A11" s="264"/>
+      <c r="B11" s="269"/>
+      <c r="C11" s="270"/>
       <c r="D11" s="135">
         <v>284</v>
       </c>
@@ -3809,10 +3809,10 @@
         <v>4.1856303808885986</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A12" s="273"/>
-      <c r="B12" s="263"/>
-      <c r="C12" s="264"/>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A12" s="264"/>
+      <c r="B12" s="269"/>
+      <c r="C12" s="270"/>
       <c r="D12" s="135">
         <v>329</v>
       </c>
@@ -3855,10 +3855,10 @@
         <v>4.1856303808885986</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A13" s="273"/>
-      <c r="B13" s="263"/>
-      <c r="C13" s="264"/>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A13" s="264"/>
+      <c r="B13" s="269"/>
+      <c r="C13" s="270"/>
       <c r="D13" s="135">
         <v>361</v>
       </c>
@@ -3902,10 +3902,10 @@
       </c>
       <c r="O13" s="132"/>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A14" s="273"/>
-      <c r="B14" s="263"/>
-      <c r="C14" s="264"/>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A14" s="264"/>
+      <c r="B14" s="269"/>
+      <c r="C14" s="270"/>
       <c r="D14" s="135">
         <v>388</v>
       </c>
@@ -3952,8 +3952,8 @@
       <c r="T14" s="38"/>
       <c r="U14" s="38"/>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A15" s="273"/>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A15" s="264"/>
       <c r="B15" s="134"/>
       <c r="C15" s="134"/>
       <c r="D15" s="134"/>
@@ -3974,28 +3974,28 @@
         <v>132</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A16" s="273"/>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A16" s="264"/>
       <c r="B16" s="161"/>
       <c r="C16" s="161"/>
       <c r="D16" s="152" t="s">
         <v>133</v>
       </c>
-      <c r="E16" s="265" t="s">
+      <c r="E16" s="271" t="s">
         <v>134</v>
       </c>
-      <c r="F16" s="266"/>
-      <c r="G16" s="266"/>
-      <c r="H16" s="266"/>
-      <c r="I16" s="266"/>
-      <c r="J16" s="266"/>
-      <c r="K16" s="266"/>
-      <c r="L16" s="266"/>
-      <c r="M16" s="266"/>
-      <c r="N16" s="267"/>
-    </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A17" s="273"/>
+      <c r="F16" s="272"/>
+      <c r="G16" s="272"/>
+      <c r="H16" s="272"/>
+      <c r="I16" s="272"/>
+      <c r="J16" s="272"/>
+      <c r="K16" s="272"/>
+      <c r="L16" s="272"/>
+      <c r="M16" s="272"/>
+      <c r="N16" s="273"/>
+    </row>
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A17" s="264"/>
       <c r="B17" s="134"/>
       <c r="C17" s="134"/>
       <c r="E17" s="162"/>
@@ -4003,8 +4003,8 @@
       <c r="G17" s="163"/>
       <c r="N17" s="164"/>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A18" s="273"/>
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A18" s="264"/>
       <c r="B18" s="134"/>
       <c r="C18" s="134"/>
       <c r="E18" s="162"/>
@@ -4015,46 +4015,46 @@
         <v>135</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A19" s="273"/>
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A19" s="264"/>
       <c r="B19" s="134"/>
       <c r="C19" s="134"/>
       <c r="E19" s="38"/>
       <c r="F19" s="38"/>
       <c r="N19" s="164"/>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A20" s="273"/>
+    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A20" s="264"/>
       <c r="B20" s="161"/>
       <c r="C20" s="161"/>
-      <c r="D20" s="268" t="s">
+      <c r="D20" s="274" t="s">
         <v>136</v>
       </c>
-      <c r="E20" s="262"/>
-      <c r="F20" s="262"/>
-      <c r="G20" s="262"/>
-      <c r="H20" s="262"/>
-      <c r="I20" s="262"/>
-      <c r="J20" s="262"/>
-      <c r="K20" s="262"/>
-      <c r="L20" s="262"/>
-      <c r="M20" s="262"/>
-      <c r="N20" s="262"/>
-      <c r="O20" s="262"/>
-      <c r="P20" s="262"/>
-      <c r="Q20" s="262"/>
-      <c r="R20" s="262"/>
-      <c r="S20" s="262"/>
-      <c r="T20" s="262"/>
-      <c r="U20" s="262"/>
-      <c r="V20" s="262"/>
-      <c r="W20" s="262"/>
-      <c r="X20" s="262"/>
-      <c r="Y20" s="262"/>
-      <c r="Z20" s="262"/>
-    </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A21" s="273"/>
+      <c r="E20" s="268"/>
+      <c r="F20" s="268"/>
+      <c r="G20" s="268"/>
+      <c r="H20" s="268"/>
+      <c r="I20" s="268"/>
+      <c r="J20" s="268"/>
+      <c r="K20" s="268"/>
+      <c r="L20" s="268"/>
+      <c r="M20" s="268"/>
+      <c r="N20" s="268"/>
+      <c r="O20" s="268"/>
+      <c r="P20" s="268"/>
+      <c r="Q20" s="268"/>
+      <c r="R20" s="268"/>
+      <c r="S20" s="268"/>
+      <c r="T20" s="268"/>
+      <c r="U20" s="268"/>
+      <c r="V20" s="268"/>
+      <c r="W20" s="268"/>
+      <c r="X20" s="268"/>
+      <c r="Y20" s="268"/>
+      <c r="Z20" s="268"/>
+    </row>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A21" s="264"/>
       <c r="B21" s="134"/>
       <c r="C21" s="134"/>
       <c r="D21" s="165"/>
@@ -4070,8 +4070,8 @@
       <c r="N21" s="167"/>
       <c r="O21" s="165"/>
     </row>
-    <row r="22" spans="1:28" s="10" customFormat="1" ht="150" x14ac:dyDescent="0.2">
-      <c r="A22" s="274"/>
+    <row r="22" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
+      <c r="A22" s="265"/>
       <c r="B22" s="9" t="s">
         <v>82</v>
       </c>
@@ -4154,10 +4154,10 @@
         <v>129</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="269"/>
-      <c r="B23" s="269"/>
-      <c r="C23" s="269"/>
+    <row r="23" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="260"/>
+      <c r="B23" s="260"/>
+      <c r="C23" s="260"/>
       <c r="D23" s="135">
         <v>12</v>
       </c>
@@ -4237,12 +4237,12 @@
         <f>Aerodinamika!G31</f>
         <v>1.2973599999999996</v>
       </c>
-      <c r="AB23" s="260"/>
-    </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A24" s="270"/>
-      <c r="B24" s="270"/>
-      <c r="C24" s="270"/>
+      <c r="AB23" s="266"/>
+    </row>
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A24" s="261"/>
+      <c r="B24" s="261"/>
+      <c r="C24" s="261"/>
       <c r="D24" s="135">
         <v>39</v>
       </c>
@@ -4315,12 +4315,12 @@
         <f>O23*X24</f>
         <v>0.34740732161375365</v>
       </c>
-      <c r="AB24" s="261"/>
-    </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A25" s="270"/>
-      <c r="B25" s="270"/>
-      <c r="C25" s="270"/>
+      <c r="AB24" s="267"/>
+    </row>
+    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A25" s="261"/>
+      <c r="B25" s="261"/>
+      <c r="C25" s="261"/>
       <c r="D25" s="152">
         <v>71</v>
       </c>
@@ -4358,10 +4358,10 @@
       <c r="R25" s="157"/>
       <c r="S25" s="157"/>
     </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A26" s="270"/>
-      <c r="B26" s="270"/>
-      <c r="C26" s="270"/>
+    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A26" s="261"/>
+      <c r="B26" s="261"/>
+      <c r="C26" s="261"/>
       <c r="D26" s="135">
         <v>116</v>
       </c>
@@ -4403,10 +4403,10 @@
         <v>130</v>
       </c>
     </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A27" s="270"/>
-      <c r="B27" s="270"/>
-      <c r="C27" s="270"/>
+    <row r="27" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A27" s="261"/>
+      <c r="B27" s="261"/>
+      <c r="C27" s="261"/>
       <c r="D27" s="135">
         <v>200</v>
       </c>
@@ -4437,10 +4437,10 @@
         <v>4.1856303808885986</v>
       </c>
     </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A28" s="270"/>
-      <c r="B28" s="270"/>
-      <c r="C28" s="270"/>
+    <row r="28" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A28" s="261"/>
+      <c r="B28" s="261"/>
+      <c r="C28" s="261"/>
       <c r="D28" s="135">
         <v>284</v>
       </c>
@@ -4471,10 +4471,10 @@
         <v>4.1856303808885986</v>
       </c>
     </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A29" s="270"/>
-      <c r="B29" s="270"/>
-      <c r="C29" s="270"/>
+    <row r="29" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A29" s="261"/>
+      <c r="B29" s="261"/>
+      <c r="C29" s="261"/>
       <c r="D29" s="135">
         <v>329</v>
       </c>
@@ -4505,10 +4505,10 @@
         <v>4.1856303808885986</v>
       </c>
     </row>
-    <row r="30" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A30" s="270"/>
-      <c r="B30" s="270"/>
-      <c r="C30" s="270"/>
+    <row r="30" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A30" s="261"/>
+      <c r="B30" s="261"/>
+      <c r="C30" s="261"/>
       <c r="D30" s="135">
         <v>361</v>
       </c>
@@ -4540,10 +4540,10 @@
       </c>
       <c r="O30" s="132"/>
     </row>
-    <row r="31" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A31" s="271"/>
-      <c r="B31" s="271"/>
-      <c r="C31" s="271"/>
+    <row r="31" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A31" s="262"/>
+      <c r="B31" s="262"/>
+      <c r="C31" s="262"/>
       <c r="D31" s="135">
         <v>388</v>
       </c>
@@ -4581,16 +4581,16 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="ecyaGde8bRCGGLjxH6/y64hd/Qu1QGpziWOApJzf8uG7KOwveh+XtxYm7qcvHDbOm4wNpJpjwTw6EQ3sZyT0Ww==" saltValue="0y2ywmKlSNb5pUNmtC6Umw==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="11">
+    <mergeCell ref="D3:Z3"/>
+    <mergeCell ref="B6:B14"/>
+    <mergeCell ref="C6:C14"/>
+    <mergeCell ref="AB6:AB7"/>
+    <mergeCell ref="E16:N16"/>
     <mergeCell ref="A23:A31"/>
     <mergeCell ref="B23:B31"/>
     <mergeCell ref="C23:C31"/>
     <mergeCell ref="A6:A22"/>
     <mergeCell ref="AB23:AB24"/>
-    <mergeCell ref="D3:Z3"/>
-    <mergeCell ref="B6:B14"/>
-    <mergeCell ref="C6:C14"/>
-    <mergeCell ref="AB6:AB7"/>
-    <mergeCell ref="E16:N16"/>
     <mergeCell ref="D20:Z20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4600,21 +4600,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B782CE6F-4AAF-42E1-A4E9-B039A4011BD6}">
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" style="39" customWidth="1"/>
-    <col min="2" max="2" width="8.42578125" style="39" customWidth="1"/>
-    <col min="3" max="4" width="9.140625" style="39"/>
-    <col min="5" max="5" width="10.7109375" style="39" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="39"/>
-    <col min="7" max="7" width="11.28515625" style="39" customWidth="1"/>
-    <col min="8" max="8" width="12.140625" style="39" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" style="39" customWidth="1"/>
-    <col min="10" max="10" width="10.5703125" style="39" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="39"/>
+    <col min="1" max="1" width="12.453125" style="39" customWidth="1"/>
+    <col min="2" max="2" width="8.453125" style="39" customWidth="1"/>
+    <col min="3" max="4" width="9.1796875" style="39"/>
+    <col min="5" max="5" width="10.7265625" style="39" customWidth="1"/>
+    <col min="6" max="6" width="9.1796875" style="39"/>
+    <col min="7" max="7" width="11.26953125" style="39" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" style="39" customWidth="1"/>
+    <col min="9" max="9" width="10.81640625" style="39" customWidth="1"/>
+    <col min="10" max="10" width="10.54296875" style="39" customWidth="1"/>
+    <col min="11" max="16384" width="9.1796875" style="39"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="15" x14ac:dyDescent="0.3">
       <c r="A1" s="38"/>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -4625,7 +4625,7 @@
       <c r="H1" s="10"/>
       <c r="I1" s="10"/>
     </row>
-    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="15" x14ac:dyDescent="0.3">
       <c r="A2" s="40"/>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -4636,7 +4636,7 @@
       <c r="H2" s="10"/>
       <c r="I2" s="10"/>
     </row>
-    <row r="3" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="275" t="s">
         <v>108</v>
       </c>
@@ -4650,7 +4650,7 @@
       <c r="I3" s="275"/>
       <c r="J3" s="275"/>
     </row>
-    <row r="4" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="14" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -4661,7 +4661,7 @@
       <c r="H4" s="10"/>
       <c r="I4" s="10"/>
     </row>
-    <row r="5" spans="1:12" ht="90" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="84" x14ac:dyDescent="0.3">
       <c r="A5" s="9"/>
       <c r="B5" s="9" t="s">
         <v>37</v>
@@ -4697,7 +4697,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="41"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -4711,7 +4711,7 @@
       <c r="K6" s="46"/>
       <c r="L6" s="46"/>
     </row>
-    <row r="7" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="41" t="s">
         <v>25</v>
       </c>
@@ -4752,7 +4752,7 @@
       </c>
       <c r="L7" s="46"/>
     </row>
-    <row r="8" spans="1:12" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ht="15" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
       <c r="B8" s="81"/>
       <c r="C8" s="82"/>
@@ -4766,7 +4766,7 @@
       <c r="K8" s="46"/>
       <c r="L8" s="46"/>
     </row>
-    <row r="9" spans="1:12" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" ht="15" x14ac:dyDescent="0.3">
       <c r="A9" s="13"/>
       <c r="B9" s="81"/>
       <c r="C9" s="82"/>
@@ -4780,7 +4780,7 @@
       <c r="K9" s="46"/>
       <c r="L9" s="46"/>
     </row>
-    <row r="10" spans="1:12" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="86"/>
       <c r="B10" s="81"/>
       <c r="C10" s="13"/>
@@ -4794,7 +4794,7 @@
       <c r="K10" s="46"/>
       <c r="L10" s="46"/>
     </row>
-    <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H11" s="276" t="s">
         <v>30</v>
       </c>
@@ -4802,54 +4802,54 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H12" s="277"/>
       <c r="I12" s="280"/>
     </row>
-    <row r="13" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H13" s="277"/>
       <c r="I13" s="280"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="H14" s="277"/>
       <c r="I14" s="280"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="H15" s="277"/>
       <c r="I15" s="280"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="H16" s="277"/>
       <c r="I16" s="280"/>
     </row>
-    <row r="17" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H17" s="277"/>
       <c r="I17" s="280"/>
     </row>
-    <row r="18" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H18" s="278"/>
       <c r="I18" s="280"/>
     </row>
-    <row r="19" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I19" s="280"/>
     </row>
-    <row r="20" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I20" s="281"/>
     </row>
-    <row r="21" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I21" s="57"/>
     </row>
-    <row r="22" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="23" spans="8:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="22" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="23" spans="8:9" ht="14" x14ac:dyDescent="0.3">
       <c r="I23" s="56"/>
     </row>
-    <row r="24" spans="8:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="24" spans="8:9" ht="14" x14ac:dyDescent="0.3">
       <c r="I24" s="56"/>
     </row>
-    <row r="25" spans="8:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="25" spans="8:9" ht="14" x14ac:dyDescent="0.3">
       <c r="I25" s="56"/>
     </row>
-    <row r="26" spans="8:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="26" spans="8:9" ht="14" x14ac:dyDescent="0.3">
       <c r="I26" s="56"/>
     </row>
   </sheetData>
@@ -4869,36 +4869,36 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Y81"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="13.28515625" style="14" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" style="14" customWidth="1"/>
-    <col min="4" max="4" width="11.140625" style="14" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" style="14" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" style="14" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" style="14" customWidth="1"/>
-    <col min="8" max="8" width="9.85546875" style="14" customWidth="1"/>
-    <col min="9" max="9" width="8.85546875" style="14" customWidth="1"/>
-    <col min="10" max="10" width="10.5703125" style="14" customWidth="1"/>
-    <col min="11" max="11" width="10.42578125" style="14" customWidth="1"/>
-    <col min="12" max="12" width="11.85546875" style="14" customWidth="1"/>
-    <col min="13" max="13" width="9.85546875" style="14" customWidth="1"/>
-    <col min="14" max="14" width="11.7109375" style="14" customWidth="1"/>
-    <col min="15" max="15" width="12.85546875" style="14" customWidth="1"/>
-    <col min="16" max="16" width="6.5703125" style="14" customWidth="1"/>
-    <col min="17" max="17" width="7.7109375" style="14" customWidth="1"/>
-    <col min="18" max="18" width="17.5703125" style="14" customWidth="1"/>
-    <col min="19" max="19" width="15.28515625" style="14" customWidth="1"/>
-    <col min="20" max="20" width="10.42578125" style="14" customWidth="1"/>
-    <col min="21" max="21" width="11.140625" style="14" customWidth="1"/>
-    <col min="22" max="22" width="13.42578125" style="14" customWidth="1"/>
-    <col min="23" max="23" width="5.140625" style="14" customWidth="1"/>
-    <col min="24" max="24" width="11.7109375" style="14" customWidth="1"/>
-    <col min="25" max="25" width="10.28515625" style="14" customWidth="1"/>
-    <col min="26" max="16384" width="9.140625" style="14"/>
+    <col min="1" max="2" width="13.26953125" style="14" customWidth="1"/>
+    <col min="3" max="3" width="26.1796875" style="14" customWidth="1"/>
+    <col min="4" max="4" width="11.1796875" style="14" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" style="14" customWidth="1"/>
+    <col min="6" max="6" width="13.7265625" style="14" customWidth="1"/>
+    <col min="7" max="7" width="10.81640625" style="14" customWidth="1"/>
+    <col min="8" max="8" width="9.81640625" style="14" customWidth="1"/>
+    <col min="9" max="9" width="8.81640625" style="14" customWidth="1"/>
+    <col min="10" max="10" width="10.54296875" style="14" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" style="14" customWidth="1"/>
+    <col min="12" max="12" width="11.81640625" style="14" customWidth="1"/>
+    <col min="13" max="13" width="9.81640625" style="14" customWidth="1"/>
+    <col min="14" max="14" width="11.7265625" style="14" customWidth="1"/>
+    <col min="15" max="15" width="12.81640625" style="14" customWidth="1"/>
+    <col min="16" max="16" width="6.54296875" style="14" customWidth="1"/>
+    <col min="17" max="17" width="7.7265625" style="14" customWidth="1"/>
+    <col min="18" max="18" width="17.54296875" style="14" customWidth="1"/>
+    <col min="19" max="19" width="15.26953125" style="14" customWidth="1"/>
+    <col min="20" max="20" width="10.453125" style="14" customWidth="1"/>
+    <col min="21" max="21" width="11.1796875" style="14" customWidth="1"/>
+    <col min="22" max="22" width="13.453125" style="14" customWidth="1"/>
+    <col min="23" max="23" width="5.1796875" style="14" customWidth="1"/>
+    <col min="24" max="24" width="11.7265625" style="14" customWidth="1"/>
+    <col min="25" max="25" width="10.26953125" style="14" customWidth="1"/>
+    <col min="26" max="16384" width="9.1796875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C1" s="287" t="s">
         <v>18</v>
       </c>
@@ -4906,7 +4906,7 @@
       <c r="E1" s="15"/>
       <c r="S1" s="16"/>
     </row>
-    <row r="2" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="288" t="s">
         <v>100</v>
       </c>
@@ -4929,7 +4929,7 @@
       <c r="R2" s="288"/>
       <c r="S2" s="288"/>
     </row>
-    <row r="3" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
       <c r="B3" s="17"/>
       <c r="C3" s="18"/>
@@ -4950,10 +4950,10 @@
       <c r="R3" s="18"/>
       <c r="S3" s="18"/>
     </row>
-    <row r="4" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="T4" s="28"/>
     </row>
-    <row r="5" spans="1:25" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="100.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>8</v>
       </c>
@@ -5027,7 +5027,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="15.5" x14ac:dyDescent="0.3">
       <c r="A6" s="184" t="str">
         <f>Greitis!A6</f>
         <v>XXXX-XX-XX</v>
@@ -5112,7 +5112,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" s="37"/>
       <c r="B7" s="34"/>
       <c r="C7" s="284"/>
@@ -5183,7 +5183,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8" s="37"/>
       <c r="B8" s="34"/>
       <c r="C8" s="284"/>
@@ -5254,7 +5254,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9" s="49"/>
       <c r="B9" s="49"/>
       <c r="C9" s="284"/>
@@ -5328,7 +5328,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="49"/>
       <c r="B10" s="49"/>
       <c r="C10" s="284"/>
@@ -5399,7 +5399,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11" s="49"/>
       <c r="B11" s="49"/>
       <c r="C11" s="284"/>
@@ -5464,7 +5464,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="49"/>
       <c r="B12" s="49"/>
       <c r="C12" s="284"/>
@@ -5529,7 +5529,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="49"/>
       <c r="B13" s="49"/>
       <c r="C13" s="284"/>
@@ -5591,7 +5591,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="36"/>
       <c r="B14" s="36"/>
       <c r="C14" s="285"/>
@@ -5653,7 +5653,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
       <c r="L15" s="70">
         <f>SUM(L6:L14)</f>
         <v>0.44999999999999996</v>
@@ -5667,7 +5667,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L16" s="68" t="s">
         <v>29</v>
       </c>
@@ -5678,12 +5678,12 @@
         <v>137</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A19" s="184" t="str">
         <f t="shared" ref="A19:I19" si="27">(A6)</f>
         <v>XXXX-XX-XX</v>
@@ -5765,7 +5765,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A20" s="37"/>
       <c r="B20" s="34"/>
       <c r="C20" s="284"/>
@@ -5827,7 +5827,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A21" s="37"/>
       <c r="B21" s="34"/>
       <c r="C21" s="284"/>
@@ -5889,7 +5889,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A22" s="49"/>
       <c r="B22" s="49"/>
       <c r="C22" s="284"/>
@@ -5951,7 +5951,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A23" s="49"/>
       <c r="B23" s="49"/>
       <c r="C23" s="284"/>
@@ -6013,7 +6013,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A24" s="49"/>
       <c r="B24" s="49"/>
       <c r="C24" s="284"/>
@@ -6075,7 +6075,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A25" s="49"/>
       <c r="B25" s="49"/>
       <c r="C25" s="284"/>
@@ -6137,7 +6137,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A26" s="49"/>
       <c r="B26" s="49"/>
       <c r="C26" s="284"/>
@@ -6199,7 +6199,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A27" s="36"/>
       <c r="B27" s="36"/>
       <c r="C27" s="285"/>
@@ -6261,7 +6261,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.3">
       <c r="L28" s="70">
         <f>SUM(L19:L27)</f>
         <v>0.44999999999999996</v>
@@ -6275,7 +6275,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:25" ht="28" x14ac:dyDescent="0.3">
       <c r="L29" s="68" t="s">
         <v>29</v>
       </c>
@@ -6286,7 +6286,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="31" spans="1:25" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:25" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L31" s="67"/>
       <c r="M31" s="123">
         <f>(M15+M28)</f>
@@ -6300,7 +6300,7 @@
       <c r="P31" s="96"/>
       <c r="Q31" s="96"/>
     </row>
-    <row r="32" spans="1:25" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:25" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L32" s="67"/>
       <c r="M32" s="45" t="s">
         <v>99</v>
@@ -6309,20 +6309,20 @@
         <v>138</v>
       </c>
     </row>
-    <row r="41" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" s="25"/>
       <c r="B78" s="25"/>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" s="25"/>
       <c r="B79" s="25"/>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" s="25"/>
       <c r="B80" s="25"/>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" s="25"/>
       <c r="B81" s="25"/>
     </row>
@@ -6353,33 +6353,33 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q263"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" style="14" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="14" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" style="14" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" style="14" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="14" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" style="14" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" style="14" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" style="14" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" style="14" customWidth="1" outlineLevel="1"/>
+    <col min="1" max="1" width="11.26953125" style="14" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" style="14" customWidth="1"/>
+    <col min="3" max="3" width="20.81640625" style="14" customWidth="1"/>
+    <col min="4" max="4" width="12.81640625" style="14" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" style="14" customWidth="1"/>
+    <col min="6" max="6" width="16.7265625" style="14" customWidth="1"/>
+    <col min="7" max="7" width="13.54296875" style="14" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" style="14" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" style="14" customWidth="1" outlineLevel="1"/>
     <col min="10" max="10" width="10" style="14" customWidth="1" outlineLevel="1"/>
-    <col min="11" max="11" width="10.28515625" style="14" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" style="14" customWidth="1"/>
+    <col min="11" max="11" width="10.26953125" style="14" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" style="14" customWidth="1"/>
     <col min="13" max="13" width="17" style="14" customWidth="1"/>
-    <col min="14" max="14" width="14.85546875" style="14" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="14"/>
+    <col min="14" max="14" width="14.81640625" style="14" customWidth="1"/>
+    <col min="15" max="16384" width="9.1796875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C1" s="287" t="s">
         <v>19</v>
       </c>
       <c r="D1" s="287"/>
       <c r="Q1" s="16"/>
     </row>
-    <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C2" s="289" t="s">
         <v>101</v>
       </c>
@@ -6395,13 +6395,13 @@
       <c r="M2" s="289"/>
       <c r="Q2" s="16"/>
     </row>
-    <row r="3" spans="1:17" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C3" s="24"/>
       <c r="H3" s="25"/>
       <c r="Q3" s="16"/>
     </row>
-    <row r="4" spans="1:17" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:17" ht="126.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" ht="8.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:17" ht="126.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="99" t="s">
         <v>8</v>
       </c>
@@ -6445,7 +6445,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="191" t="str">
         <f>Paėmimas!A6</f>
         <v>XXXX-XX-XX</v>
@@ -6503,7 +6503,7 @@
         <v>1 linija, 1 filtras</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="59"/>
       <c r="B7" s="23"/>
       <c r="C7" s="284"/>
@@ -6540,7 +6540,7 @@
       <c r="M7" s="60"/>
       <c r="N7" s="34"/>
     </row>
-    <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="59"/>
       <c r="B8" s="23"/>
       <c r="C8" s="284"/>
@@ -6577,7 +6577,7 @@
       <c r="M8" s="60"/>
       <c r="N8" s="34"/>
     </row>
-    <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="59"/>
       <c r="B9" s="23"/>
       <c r="C9" s="284"/>
@@ -6614,7 +6614,7 @@
       <c r="M9" s="60"/>
       <c r="N9" s="34"/>
     </row>
-    <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="59"/>
       <c r="B10" s="23"/>
       <c r="C10" s="284"/>
@@ -6651,7 +6651,7 @@
       <c r="M10" s="60"/>
       <c r="N10" s="34"/>
     </row>
-    <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="59"/>
       <c r="B11" s="23"/>
       <c r="C11" s="284"/>
@@ -6688,7 +6688,7 @@
       <c r="M11" s="60"/>
       <c r="N11" s="34"/>
     </row>
-    <row r="12" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="59"/>
       <c r="B12" s="23"/>
       <c r="C12" s="284"/>
@@ -6725,7 +6725,7 @@
       <c r="M12" s="60"/>
       <c r="N12" s="34"/>
     </row>
-    <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="59"/>
       <c r="B13" s="23"/>
       <c r="C13" s="284"/>
@@ -6762,7 +6762,7 @@
       <c r="M13" s="60"/>
       <c r="N13" s="34"/>
     </row>
-    <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="61"/>
       <c r="B14" s="62"/>
       <c r="C14" s="285"/>
@@ -6799,7 +6799,7 @@
       <c r="M14" s="63"/>
       <c r="N14" s="22"/>
     </row>
-    <row r="15" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C15" s="78"/>
       <c r="D15" s="78"/>
       <c r="E15" s="78"/>
@@ -6815,7 +6815,7 @@
       </c>
       <c r="J15" s="78"/>
     </row>
-    <row r="16" spans="1:17" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C16" s="79"/>
       <c r="D16" s="79"/>
       <c r="E16" s="79"/>
@@ -6829,7 +6829,7 @@
       </c>
       <c r="J16" s="79"/>
     </row>
-    <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C17" s="79"/>
       <c r="D17" s="79"/>
       <c r="E17" s="79"/>
@@ -6839,7 +6839,7 @@
       <c r="I17" s="79"/>
       <c r="J17" s="79"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="191" t="str">
         <f>Paėmimas!A19</f>
         <v>XXXX-XX-XX</v>
@@ -6897,7 +6897,7 @@
         <v>2 linija, 2 filtras</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="59"/>
       <c r="B20" s="23"/>
       <c r="C20" s="284"/>
@@ -6934,7 +6934,7 @@
       <c r="M20" s="60"/>
       <c r="N20" s="34"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="59"/>
       <c r="B21" s="23"/>
       <c r="C21" s="284"/>
@@ -6971,7 +6971,7 @@
       <c r="M21" s="60"/>
       <c r="N21" s="34"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="59"/>
       <c r="B22" s="23"/>
       <c r="C22" s="284"/>
@@ -7008,7 +7008,7 @@
       <c r="M22" s="60"/>
       <c r="N22" s="34"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="59"/>
       <c r="B23" s="23"/>
       <c r="C23" s="284"/>
@@ -7045,7 +7045,7 @@
       <c r="M23" s="60"/>
       <c r="N23" s="34"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="59"/>
       <c r="B24" s="23"/>
       <c r="C24" s="284"/>
@@ -7082,7 +7082,7 @@
       <c r="M24" s="60"/>
       <c r="N24" s="34"/>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="59"/>
       <c r="B25" s="23"/>
       <c r="C25" s="284"/>
@@ -7119,7 +7119,7 @@
       <c r="M25" s="60"/>
       <c r="N25" s="34"/>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="59"/>
       <c r="B26" s="23"/>
       <c r="C26" s="284"/>
@@ -7156,7 +7156,7 @@
       <c r="M26" s="60"/>
       <c r="N26" s="34"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="61"/>
       <c r="B27" s="62"/>
       <c r="C27" s="285"/>
@@ -7193,7 +7193,7 @@
       <c r="M27" s="63"/>
       <c r="N27" s="22"/>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C28" s="78"/>
       <c r="D28" s="78"/>
       <c r="E28" s="78"/>
@@ -7216,7 +7216,7 @@
         <v>1.0353315592396999</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" ht="56" x14ac:dyDescent="0.3">
       <c r="C29" s="79"/>
       <c r="D29" s="79"/>
       <c r="E29" s="79"/>
@@ -7235,7 +7235,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C30" s="80"/>
       <c r="D30" s="80"/>
       <c r="E30" s="80"/>
@@ -7245,7 +7245,7 @@
       <c r="I30" s="80"/>
       <c r="J30" s="80"/>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C31" s="80"/>
       <c r="D31" s="80"/>
       <c r="E31" s="80"/>
@@ -7261,7 +7261,7 @@
       </c>
       <c r="J31" s="80"/>
     </row>
-    <row r="32" spans="1:14" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C32" s="80"/>
       <c r="D32" s="80"/>
       <c r="E32" s="80"/>
@@ -7275,7 +7275,7 @@
       </c>
       <c r="J32" s="80"/>
     </row>
-    <row r="33" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C33" s="80"/>
       <c r="D33" s="80"/>
       <c r="E33" s="80"/>
@@ -7285,7 +7285,7 @@
       <c r="I33" s="80"/>
       <c r="J33" s="80"/>
     </row>
-    <row r="34" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:10" x14ac:dyDescent="0.3">
       <c r="C34" s="80"/>
       <c r="D34" s="80"/>
       <c r="E34" s="80"/>
@@ -7295,13 +7295,13 @@
       <c r="I34" s="80"/>
       <c r="J34" s="80"/>
     </row>
-    <row r="262" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="262" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C262" s="26"/>
       <c r="D262" s="14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="263" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="263" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C263" s="27"/>
       <c r="D263" s="14" t="s">
         <v>11</v>
@@ -7331,36 +7331,36 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:R8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="14" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" style="14" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" style="14" customWidth="1"/>
-    <col min="4" max="4" width="8.140625" style="14" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="14" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" style="14" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" style="14" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" style="14" customWidth="1"/>
+    <col min="3" max="3" width="24.54296875" style="14" customWidth="1"/>
+    <col min="4" max="4" width="8.1796875" style="14" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" style="14" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" style="14" customWidth="1"/>
     <col min="7" max="7" width="11" style="14" customWidth="1"/>
-    <col min="8" max="9" width="10.28515625" style="14" customWidth="1"/>
-    <col min="10" max="10" width="11.140625" style="14" customWidth="1"/>
-    <col min="11" max="11" width="14.28515625" style="14" customWidth="1"/>
-    <col min="12" max="12" width="11.28515625" style="14" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" style="14" customWidth="1"/>
-    <col min="14" max="14" width="17.7109375" style="14" customWidth="1"/>
-    <col min="15" max="15" width="8.28515625" style="14" customWidth="1"/>
-    <col min="16" max="16" width="12.7109375" style="14" customWidth="1"/>
-    <col min="17" max="17" width="9.140625" style="14"/>
-    <col min="18" max="18" width="9.5703125" style="14" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.140625" style="14"/>
+    <col min="8" max="9" width="10.26953125" style="14" customWidth="1"/>
+    <col min="10" max="10" width="11.1796875" style="14" customWidth="1"/>
+    <col min="11" max="11" width="14.26953125" style="14" customWidth="1"/>
+    <col min="12" max="12" width="11.26953125" style="14" customWidth="1"/>
+    <col min="13" max="13" width="10.54296875" style="14" customWidth="1"/>
+    <col min="14" max="14" width="17.7265625" style="14" customWidth="1"/>
+    <col min="15" max="15" width="8.26953125" style="14" customWidth="1"/>
+    <col min="16" max="16" width="12.7265625" style="14" customWidth="1"/>
+    <col min="17" max="17" width="9.1796875" style="14"/>
+    <col min="18" max="18" width="9.54296875" style="14" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.1796875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C1" s="287" t="s">
         <v>20</v>
       </c>
       <c r="D1" s="287"/>
       <c r="R1" s="16"/>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="289" t="s">
         <v>102</v>
       </c>
@@ -7379,16 +7379,16 @@
       <c r="N2" s="289"/>
       <c r="O2" s="125"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="F3" s="29"/>
       <c r="L3" s="16"/>
       <c r="M3" s="16"/>
     </row>
-    <row r="4" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="L4" s="16"/>
       <c r="M4" s="16"/>
     </row>
-    <row r="5" spans="1:18" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="88.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="99" t="s">
         <v>8</v>
       </c>
@@ -7438,7 +7438,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="196" t="str">
         <f>Paėmimas!A6</f>
         <v>XXXX-XX-XX</v>
@@ -7503,7 +7503,7 @@
         <v>1 linija, 1 filtras</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="207"/>
       <c r="B7" s="208"/>
       <c r="C7" s="290"/>
@@ -7551,7 +7551,7 @@
         <v>2 linija, 2 filtras</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="209"/>
       <c r="B8" s="210"/>
       <c r="C8" s="291"/>
@@ -7589,27 +7589,27 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{330ECBA1-822C-4C0F-89AB-CB2C7AD5643F}">
   <dimension ref="A1:P18"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" style="95" customWidth="1"/>
-    <col min="2" max="2" width="25.140625" style="95" customWidth="1"/>
-    <col min="3" max="3" width="7.42578125" style="95" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" style="95" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" style="95" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" style="95" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" style="95" customWidth="1"/>
+    <col min="1" max="1" width="13.7265625" style="95" customWidth="1"/>
+    <col min="2" max="2" width="25.1796875" style="95" customWidth="1"/>
+    <col min="3" max="3" width="7.453125" style="95" customWidth="1"/>
+    <col min="4" max="4" width="12.81640625" style="95" customWidth="1"/>
+    <col min="5" max="5" width="11.1796875" style="95" customWidth="1"/>
+    <col min="6" max="6" width="10.81640625" style="95" customWidth="1"/>
+    <col min="7" max="7" width="10.453125" style="95" customWidth="1"/>
     <col min="8" max="8" width="18" style="95" customWidth="1"/>
-    <col min="9" max="9" width="11.28515625" style="95" customWidth="1"/>
-    <col min="10" max="10" width="10.85546875" style="95" customWidth="1"/>
+    <col min="9" max="9" width="11.26953125" style="95" customWidth="1"/>
+    <col min="10" max="10" width="10.81640625" style="95" customWidth="1"/>
     <col min="11" max="11" width="11" style="95" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" style="95" customWidth="1"/>
-    <col min="13" max="13" width="20.28515625" style="95" customWidth="1"/>
-    <col min="14" max="14" width="16.85546875" style="95" customWidth="1"/>
-    <col min="15" max="15" width="31.28515625" style="95" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="95"/>
+    <col min="12" max="12" width="11.1796875" style="95" customWidth="1"/>
+    <col min="13" max="13" width="20.26953125" style="95" customWidth="1"/>
+    <col min="14" max="14" width="16.81640625" style="95" customWidth="1"/>
+    <col min="15" max="15" width="31.26953125" style="95" customWidth="1"/>
+    <col min="16" max="16384" width="9.1796875" style="95"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C1" s="287" t="s">
         <v>21</v>
       </c>
@@ -7617,7 +7617,7 @@
       <c r="E1" s="287"/>
       <c r="F1" s="287"/>
     </row>
-    <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="289" t="s">
         <v>103</v>
       </c>
@@ -7636,50 +7636,50 @@
       <c r="N2" s="289"/>
       <c r="O2" s="289"/>
     </row>
-    <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="293" t="s">
+    <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="298" t="s">
         <v>82</v>
       </c>
-      <c r="B4" s="293" t="s">
+      <c r="B4" s="298" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="304" t="s">
+      <c r="C4" s="295" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="304" t="s">
+      <c r="D4" s="295" t="s">
         <v>84</v>
       </c>
-      <c r="E4" s="304" t="s">
+      <c r="E4" s="295" t="s">
         <v>85</v>
       </c>
-      <c r="F4" s="304"/>
-      <c r="G4" s="304"/>
-      <c r="H4" s="304" t="s">
+      <c r="F4" s="295"/>
+      <c r="G4" s="295"/>
+      <c r="H4" s="295" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="297" t="s">
+      <c r="I4" s="302" t="s">
         <v>86</v>
       </c>
-      <c r="J4" s="292" t="s">
+      <c r="J4" s="297" t="s">
         <v>87</v>
       </c>
-      <c r="K4" s="292"/>
-      <c r="L4" s="292"/>
-      <c r="M4" s="299" t="s">
+      <c r="K4" s="297"/>
+      <c r="L4" s="297"/>
+      <c r="M4" s="304" t="s">
         <v>88</v>
       </c>
-      <c r="N4" s="292" t="s">
+      <c r="N4" s="297" t="s">
         <v>15</v>
       </c>
-      <c r="O4" s="295" t="s">
+      <c r="O4" s="300" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="294"/>
-      <c r="B5" s="294"/>
-      <c r="C5" s="305"/>
-      <c r="D5" s="304"/>
+    <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="299"/>
+      <c r="B5" s="299"/>
+      <c r="C5" s="296"/>
+      <c r="D5" s="295"/>
       <c r="E5" s="116">
         <v>1</v>
       </c>
@@ -7689,8 +7689,8 @@
       <c r="G5" s="116">
         <v>3</v>
       </c>
-      <c r="H5" s="304"/>
-      <c r="I5" s="298"/>
+      <c r="H5" s="295"/>
+      <c r="I5" s="303"/>
       <c r="J5" s="12">
         <v>1</v>
       </c>
@@ -7700,16 +7700,16 @@
       <c r="L5" s="12">
         <v>3</v>
       </c>
-      <c r="M5" s="300"/>
-      <c r="N5" s="292"/>
-      <c r="O5" s="296"/>
-    </row>
-    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M5" s="305"/>
+      <c r="N5" s="297"/>
+      <c r="O5" s="301"/>
+    </row>
+    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="220" t="str">
         <f>Paėmimas!B6</f>
         <v>XX</v>
       </c>
-      <c r="B6" s="301" t="str">
+      <c r="B6" s="292" t="str">
         <f>Paėmimas!C6</f>
         <v>XXXX</v>
       </c>
@@ -7757,9 +7757,9 @@
         <v>1 linija, 1 filtras</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="34"/>
-      <c r="B7" s="302"/>
+      <c r="B7" s="293"/>
       <c r="C7" s="33">
         <v>2</v>
       </c>
@@ -7794,9 +7794,9 @@
         <v>2 linija, 2 filtras</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="34"/>
-      <c r="B8" s="302"/>
+      <c r="B8" s="293"/>
       <c r="C8" s="33"/>
       <c r="D8" s="89"/>
       <c r="E8" s="176"/>
@@ -7814,9 +7814,9 @@
       <c r="N8" s="90"/>
       <c r="O8" s="224"/>
     </row>
-    <row r="9" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A9" s="34"/>
-      <c r="B9" s="302"/>
+      <c r="B9" s="293"/>
       <c r="C9" s="33">
         <v>3</v>
       </c>
@@ -7851,9 +7851,9 @@
       </c>
       <c r="P9" s="97"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="34"/>
-      <c r="B10" s="302"/>
+      <c r="B10" s="293"/>
       <c r="C10" s="33"/>
       <c r="D10" s="89"/>
       <c r="E10" s="176"/>
@@ -7868,9 +7868,9 @@
       <c r="N10" s="90"/>
       <c r="O10" s="117"/>
     </row>
-    <row r="11" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A11" s="34"/>
-      <c r="B11" s="302"/>
+      <c r="B11" s="293"/>
       <c r="C11" s="33">
         <v>41</v>
       </c>
@@ -7904,9 +7904,9 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="34"/>
-      <c r="B12" s="302"/>
+      <c r="B12" s="293"/>
       <c r="C12" s="112" t="s">
         <v>45</v>
       </c>
@@ -7940,9 +7940,9 @@
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A13" s="34"/>
-      <c r="B13" s="302"/>
+      <c r="B13" s="293"/>
       <c r="C13" s="113" t="s">
         <v>46</v>
       </c>
@@ -7976,9 +7976,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A14" s="34"/>
-      <c r="B14" s="302"/>
+      <c r="B14" s="293"/>
       <c r="C14" s="113" t="s">
         <v>47</v>
       </c>
@@ -8012,9 +8012,9 @@
         <v>95</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A15" s="34"/>
-      <c r="B15" s="302"/>
+      <c r="B15" s="293"/>
       <c r="C15" s="114" t="s">
         <v>48</v>
       </c>
@@ -8048,9 +8048,9 @@
         <v>96</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="32.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="22"/>
-      <c r="B16" s="303"/>
+      <c r="B16" s="294"/>
       <c r="C16" s="33"/>
       <c r="D16" s="92"/>
       <c r="E16" s="21"/>
@@ -8070,10 +8070,10 @@
         <v>97</v>
       </c>
     </row>
-    <row r="17" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K17" s="96"/>
     </row>
-    <row r="18" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K18" s="96"/>
     </row>
   </sheetData>
@@ -8084,11 +8084,6 @@
     </sortState>
   </autoFilter>
   <mergeCells count="14">
-    <mergeCell ref="B6:B16"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:H5"/>
     <mergeCell ref="J4:L4"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="A2:O2"/>
@@ -8098,6 +8093,11 @@
     <mergeCell ref="O4:O5"/>
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="M4:M5"/>
+    <mergeCell ref="B6:B16"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="H4:H5"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -8114,16 +8114,16 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{813C0327-CFDD-498C-87C1-8E379F217A35}">
   <dimension ref="A3:D10"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" style="104" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" style="104" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" style="104" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" style="104" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="104"/>
+    <col min="1" max="1" width="14.7265625" style="104" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" style="104" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" style="104" customWidth="1"/>
+    <col min="4" max="4" width="21.26953125" style="104" customWidth="1"/>
+    <col min="5" max="16384" width="9.1796875" style="104"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="306" t="s">
         <v>41</v>
       </c>
@@ -8131,7 +8131,7 @@
       <c r="C3" s="306"/>
       <c r="D3" s="306"/>
     </row>
-    <row r="5" spans="1:4" ht="72.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="72.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="105" t="s">
         <v>89</v>
       </c>
@@ -8145,7 +8145,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="107">
         <f>(B6*C6*D6)/1000000</f>
         <v>1.944</v>
@@ -8160,7 +8160,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C10" s="111"/>
     </row>
   </sheetData>
@@ -8173,26 +8173,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentas" ma:contentTypeID="0x010100BAB57CF81AE55C4698AAD22D302297F0" ma:contentTypeVersion="18" ma:contentTypeDescription="Kurkite naują dokumentą." ma:contentTypeScope="" ma:versionID="49ab401eb4052690d2a2629974c22fd6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="453e7e53-5eb2-45cf-b2ab-34c867e554b8" xmlns:ns3="aa0d983d-359a-438c-9953-3af1a8ac0831" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ab9969d50e0b13c63bc5bd0499c928dc" ns2:_="" ns3:_="">
     <xsd:import namespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
@@ -8447,26 +8427,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
-    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0108C608-980F-44FC-9F17-65C384873DE6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8483,4 +8464,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Duomenų perkėlimas iš H2O į H2O ir smulkūs pataisymai
</commit_message>
<xml_diff>
--- a/PVZ1.xlsx
+++ b/PVZ1.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="155" documentId="8_{6218F508-2438-4EC7-8B4D-5D6F3C7CDB90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{201A47C8-B92F-45CF-9C07-2B82262E0461}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="3" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="2" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Compatibility Report" sheetId="4" state="hidden" r:id="rId1"/>
@@ -2719,6 +2719,38 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -2743,40 +2775,8 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -2817,6 +2817,42 @@
     <xf numFmtId="169" fontId="4" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2832,42 +2868,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -3303,31 +3303,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="D3" s="276" t="s">
+      <c r="D3" s="267" t="s">
         <v>109</v>
       </c>
-      <c r="E3" s="276"/>
-      <c r="F3" s="276"/>
-      <c r="G3" s="276"/>
-      <c r="H3" s="276"/>
-      <c r="I3" s="276"/>
-      <c r="J3" s="276"/>
-      <c r="K3" s="276"/>
-      <c r="L3" s="276"/>
-      <c r="M3" s="276"/>
-      <c r="N3" s="276"/>
-      <c r="O3" s="276"/>
-      <c r="P3" s="276"/>
-      <c r="Q3" s="276"/>
-      <c r="R3" s="276"/>
-      <c r="S3" s="276"/>
-      <c r="T3" s="276"/>
-      <c r="U3" s="276"/>
-      <c r="V3" s="276"/>
-      <c r="W3" s="276"/>
-      <c r="X3" s="276"/>
-      <c r="Y3" s="276"/>
-      <c r="Z3" s="276"/>
+      <c r="E3" s="267"/>
+      <c r="F3" s="267"/>
+      <c r="G3" s="267"/>
+      <c r="H3" s="267"/>
+      <c r="I3" s="267"/>
+      <c r="J3" s="267"/>
+      <c r="K3" s="267"/>
+      <c r="L3" s="267"/>
+      <c r="M3" s="267"/>
+      <c r="N3" s="267"/>
+      <c r="O3" s="267"/>
+      <c r="P3" s="267"/>
+      <c r="Q3" s="267"/>
+      <c r="R3" s="267"/>
+      <c r="S3" s="267"/>
+      <c r="T3" s="267"/>
+      <c r="U3" s="267"/>
+      <c r="V3" s="267"/>
+      <c r="W3" s="267"/>
+      <c r="X3" s="267"/>
+      <c r="Y3" s="267"/>
+      <c r="Z3" s="267"/>
     </row>
     <row r="5" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
@@ -3416,13 +3416,13 @@
       </c>
     </row>
     <row r="6" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="270" t="s">
+      <c r="A6" s="278" t="s">
         <v>148</v>
       </c>
-      <c r="B6" s="277" t="s">
+      <c r="B6" s="268" t="s">
         <v>147</v>
       </c>
-      <c r="C6" s="278" t="s">
+      <c r="C6" s="269" t="s">
         <v>149</v>
       </c>
       <c r="D6" s="135">
@@ -3513,14 +3513,14 @@
         <f>Aerodinamika!G31</f>
         <v>1.2973599999999996</v>
       </c>
-      <c r="AB6" s="273" t="s">
+      <c r="AB6" s="270" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="271"/>
-      <c r="B7" s="277"/>
-      <c r="C7" s="278"/>
+      <c r="A7" s="279"/>
+      <c r="B7" s="268"/>
+      <c r="C7" s="269"/>
       <c r="D7" s="135">
         <v>39</v>
       </c>
@@ -3605,12 +3605,12 @@
         <f>O6*X7</f>
         <v>0.34740732161375365</v>
       </c>
-      <c r="AB7" s="274"/>
+      <c r="AB7" s="271"/>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="271"/>
-      <c r="B8" s="277"/>
-      <c r="C8" s="278"/>
+      <c r="A8" s="279"/>
+      <c r="B8" s="268"/>
+      <c r="C8" s="269"/>
       <c r="D8" s="152">
         <v>71</v>
       </c>
@@ -3661,9 +3661,9 @@
       <c r="S8" s="157"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A9" s="271"/>
-      <c r="B9" s="277"/>
-      <c r="C9" s="278"/>
+      <c r="A9" s="279"/>
+      <c r="B9" s="268"/>
+      <c r="C9" s="269"/>
       <c r="D9" s="135">
         <v>116</v>
       </c>
@@ -3718,9 +3718,9 @@
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A10" s="271"/>
-      <c r="B10" s="277"/>
-      <c r="C10" s="278"/>
+      <c r="A10" s="279"/>
+      <c r="B10" s="268"/>
+      <c r="C10" s="269"/>
       <c r="D10" s="135">
         <v>200</v>
       </c>
@@ -3764,9 +3764,9 @@
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A11" s="271"/>
-      <c r="B11" s="277"/>
-      <c r="C11" s="278"/>
+      <c r="A11" s="279"/>
+      <c r="B11" s="268"/>
+      <c r="C11" s="269"/>
       <c r="D11" s="135">
         <v>284</v>
       </c>
@@ -3810,9 +3810,9 @@
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A12" s="271"/>
-      <c r="B12" s="277"/>
-      <c r="C12" s="278"/>
+      <c r="A12" s="279"/>
+      <c r="B12" s="268"/>
+      <c r="C12" s="269"/>
       <c r="D12" s="135">
         <v>329</v>
       </c>
@@ -3856,9 +3856,9 @@
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A13" s="271"/>
-      <c r="B13" s="277"/>
-      <c r="C13" s="278"/>
+      <c r="A13" s="279"/>
+      <c r="B13" s="268"/>
+      <c r="C13" s="269"/>
       <c r="D13" s="135">
         <v>361</v>
       </c>
@@ -3903,9 +3903,9 @@
       <c r="O13" s="132"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A14" s="271"/>
-      <c r="B14" s="277"/>
-      <c r="C14" s="278"/>
+      <c r="A14" s="279"/>
+      <c r="B14" s="268"/>
+      <c r="C14" s="269"/>
       <c r="D14" s="135">
         <v>388</v>
       </c>
@@ -3953,7 +3953,7 @@
       <c r="U14" s="38"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A15" s="271"/>
+      <c r="A15" s="279"/>
       <c r="B15" s="134"/>
       <c r="C15" s="134"/>
       <c r="D15" s="134"/>
@@ -3975,27 +3975,27 @@
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A16" s="271"/>
+      <c r="A16" s="279"/>
       <c r="B16" s="161"/>
       <c r="C16" s="161"/>
       <c r="D16" s="152" t="s">
         <v>133</v>
       </c>
-      <c r="E16" s="279" t="s">
+      <c r="E16" s="272" t="s">
         <v>134</v>
       </c>
-      <c r="F16" s="280"/>
-      <c r="G16" s="280"/>
-      <c r="H16" s="280"/>
-      <c r="I16" s="280"/>
-      <c r="J16" s="280"/>
-      <c r="K16" s="280"/>
-      <c r="L16" s="280"/>
-      <c r="M16" s="280"/>
-      <c r="N16" s="281"/>
+      <c r="F16" s="273"/>
+      <c r="G16" s="273"/>
+      <c r="H16" s="273"/>
+      <c r="I16" s="273"/>
+      <c r="J16" s="273"/>
+      <c r="K16" s="273"/>
+      <c r="L16" s="273"/>
+      <c r="M16" s="273"/>
+      <c r="N16" s="274"/>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A17" s="271"/>
+      <c r="A17" s="279"/>
       <c r="B17" s="134"/>
       <c r="C17" s="134"/>
       <c r="E17" s="162"/>
@@ -4004,7 +4004,7 @@
       <c r="N17" s="164"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A18" s="271"/>
+      <c r="A18" s="279"/>
       <c r="B18" s="134"/>
       <c r="C18" s="134"/>
       <c r="E18" s="162"/>
@@ -4016,7 +4016,7 @@
       </c>
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A19" s="271"/>
+      <c r="A19" s="279"/>
       <c r="B19" s="134"/>
       <c r="C19" s="134"/>
       <c r="E19" s="38"/>
@@ -4024,37 +4024,37 @@
       <c r="N19" s="164"/>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A20" s="271"/>
+      <c r="A20" s="279"/>
       <c r="B20" s="161"/>
       <c r="C20" s="161"/>
-      <c r="D20" s="275" t="s">
+      <c r="D20" s="281" t="s">
         <v>136</v>
       </c>
-      <c r="E20" s="276"/>
-      <c r="F20" s="276"/>
-      <c r="G20" s="276"/>
-      <c r="H20" s="276"/>
-      <c r="I20" s="276"/>
-      <c r="J20" s="276"/>
-      <c r="K20" s="276"/>
-      <c r="L20" s="276"/>
-      <c r="M20" s="276"/>
-      <c r="N20" s="276"/>
-      <c r="O20" s="276"/>
-      <c r="P20" s="276"/>
-      <c r="Q20" s="276"/>
-      <c r="R20" s="276"/>
-      <c r="S20" s="276"/>
-      <c r="T20" s="276"/>
-      <c r="U20" s="276"/>
-      <c r="V20" s="276"/>
-      <c r="W20" s="276"/>
-      <c r="X20" s="276"/>
-      <c r="Y20" s="276"/>
-      <c r="Z20" s="276"/>
+      <c r="E20" s="267"/>
+      <c r="F20" s="267"/>
+      <c r="G20" s="267"/>
+      <c r="H20" s="267"/>
+      <c r="I20" s="267"/>
+      <c r="J20" s="267"/>
+      <c r="K20" s="267"/>
+      <c r="L20" s="267"/>
+      <c r="M20" s="267"/>
+      <c r="N20" s="267"/>
+      <c r="O20" s="267"/>
+      <c r="P20" s="267"/>
+      <c r="Q20" s="267"/>
+      <c r="R20" s="267"/>
+      <c r="S20" s="267"/>
+      <c r="T20" s="267"/>
+      <c r="U20" s="267"/>
+      <c r="V20" s="267"/>
+      <c r="W20" s="267"/>
+      <c r="X20" s="267"/>
+      <c r="Y20" s="267"/>
+      <c r="Z20" s="267"/>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A21" s="271"/>
+      <c r="A21" s="279"/>
       <c r="B21" s="134"/>
       <c r="C21" s="134"/>
       <c r="D21" s="165"/>
@@ -4071,7 +4071,7 @@
       <c r="O21" s="165"/>
     </row>
     <row r="22" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
-      <c r="A22" s="272"/>
+      <c r="A22" s="280"/>
       <c r="B22" s="9" t="s">
         <v>82</v>
       </c>
@@ -4155,9 +4155,9 @@
       </c>
     </row>
     <row r="23" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="267"/>
-      <c r="B23" s="267"/>
-      <c r="C23" s="267"/>
+      <c r="A23" s="275"/>
+      <c r="B23" s="275"/>
+      <c r="C23" s="275"/>
       <c r="D23" s="135">
         <v>12</v>
       </c>
@@ -4237,12 +4237,12 @@
         <f>Aerodinamika!G31</f>
         <v>1.2973599999999996</v>
       </c>
-      <c r="AB23" s="273"/>
+      <c r="AB23" s="270"/>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A24" s="268"/>
-      <c r="B24" s="268"/>
-      <c r="C24" s="268"/>
+      <c r="A24" s="276"/>
+      <c r="B24" s="276"/>
+      <c r="C24" s="276"/>
       <c r="D24" s="135">
         <v>39</v>
       </c>
@@ -4315,12 +4315,12 @@
         <f>O23*X24</f>
         <v>0.34740732161375365</v>
       </c>
-      <c r="AB24" s="274"/>
+      <c r="AB24" s="271"/>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A25" s="268"/>
-      <c r="B25" s="268"/>
-      <c r="C25" s="268"/>
+      <c r="A25" s="276"/>
+      <c r="B25" s="276"/>
+      <c r="C25" s="276"/>
       <c r="D25" s="152">
         <v>71</v>
       </c>
@@ -4359,9 +4359,9 @@
       <c r="S25" s="157"/>
     </row>
     <row r="26" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A26" s="268"/>
-      <c r="B26" s="268"/>
-      <c r="C26" s="268"/>
+      <c r="A26" s="276"/>
+      <c r="B26" s="276"/>
+      <c r="C26" s="276"/>
       <c r="D26" s="135">
         <v>116</v>
       </c>
@@ -4404,9 +4404,9 @@
       </c>
     </row>
     <row r="27" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A27" s="268"/>
-      <c r="B27" s="268"/>
-      <c r="C27" s="268"/>
+      <c r="A27" s="276"/>
+      <c r="B27" s="276"/>
+      <c r="C27" s="276"/>
       <c r="D27" s="135">
         <v>200</v>
       </c>
@@ -4438,9 +4438,9 @@
       </c>
     </row>
     <row r="28" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A28" s="268"/>
-      <c r="B28" s="268"/>
-      <c r="C28" s="268"/>
+      <c r="A28" s="276"/>
+      <c r="B28" s="276"/>
+      <c r="C28" s="276"/>
       <c r="D28" s="135">
         <v>284</v>
       </c>
@@ -4472,9 +4472,9 @@
       </c>
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A29" s="268"/>
-      <c r="B29" s="268"/>
-      <c r="C29" s="268"/>
+      <c r="A29" s="276"/>
+      <c r="B29" s="276"/>
+      <c r="C29" s="276"/>
       <c r="D29" s="135">
         <v>329</v>
       </c>
@@ -4506,9 +4506,9 @@
       </c>
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A30" s="268"/>
-      <c r="B30" s="268"/>
-      <c r="C30" s="268"/>
+      <c r="A30" s="276"/>
+      <c r="B30" s="276"/>
+      <c r="C30" s="276"/>
       <c r="D30" s="135">
         <v>361</v>
       </c>
@@ -4541,9 +4541,9 @@
       <c r="O30" s="132"/>
     </row>
     <row r="31" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A31" s="269"/>
-      <c r="B31" s="269"/>
-      <c r="C31" s="269"/>
+      <c r="A31" s="277"/>
+      <c r="B31" s="277"/>
+      <c r="C31" s="277"/>
       <c r="D31" s="135">
         <v>388</v>
       </c>
@@ -4581,17 +4581,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="ecyaGde8bRCGGLjxH6/y64hd/Qu1QGpziWOApJzf8uG7KOwveh+XtxYm7qcvHDbOm4wNpJpjwTw6EQ3sZyT0Ww==" saltValue="0y2ywmKlSNb5pUNmtC6Umw==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="11">
-    <mergeCell ref="D3:Z3"/>
-    <mergeCell ref="B6:B14"/>
-    <mergeCell ref="C6:C14"/>
-    <mergeCell ref="AB6:AB7"/>
-    <mergeCell ref="E16:N16"/>
     <mergeCell ref="A23:A31"/>
     <mergeCell ref="B23:B31"/>
     <mergeCell ref="C23:C31"/>
     <mergeCell ref="A6:A22"/>
     <mergeCell ref="AB23:AB24"/>
     <mergeCell ref="D20:Z20"/>
+    <mergeCell ref="D3:Z3"/>
+    <mergeCell ref="B6:B14"/>
+    <mergeCell ref="C6:C14"/>
+    <mergeCell ref="AB6:AB7"/>
+    <mergeCell ref="E16:N16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7637,49 +7637,49 @@
       <c r="O2" s="289"/>
     </row>
     <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="298" t="s">
+      <c r="A4" s="293" t="s">
         <v>82</v>
       </c>
-      <c r="B4" s="298" t="s">
+      <c r="B4" s="293" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="295" t="s">
+      <c r="C4" s="304" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="295" t="s">
+      <c r="D4" s="304" t="s">
         <v>84</v>
       </c>
-      <c r="E4" s="295" t="s">
+      <c r="E4" s="304" t="s">
         <v>85</v>
       </c>
-      <c r="F4" s="295"/>
-      <c r="G4" s="295"/>
-      <c r="H4" s="295" t="s">
+      <c r="F4" s="304"/>
+      <c r="G4" s="304"/>
+      <c r="H4" s="304" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="302" t="s">
+      <c r="I4" s="297" t="s">
         <v>86</v>
       </c>
-      <c r="J4" s="297" t="s">
+      <c r="J4" s="292" t="s">
         <v>87</v>
       </c>
-      <c r="K4" s="297"/>
-      <c r="L4" s="297"/>
-      <c r="M4" s="304" t="s">
+      <c r="K4" s="292"/>
+      <c r="L4" s="292"/>
+      <c r="M4" s="299" t="s">
         <v>88</v>
       </c>
-      <c r="N4" s="297" t="s">
+      <c r="N4" s="292" t="s">
         <v>15</v>
       </c>
-      <c r="O4" s="300" t="s">
+      <c r="O4" s="295" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="299"/>
-      <c r="B5" s="299"/>
-      <c r="C5" s="296"/>
-      <c r="D5" s="295"/>
+      <c r="A5" s="294"/>
+      <c r="B5" s="294"/>
+      <c r="C5" s="305"/>
+      <c r="D5" s="304"/>
       <c r="E5" s="116">
         <v>1</v>
       </c>
@@ -7689,8 +7689,8 @@
       <c r="G5" s="116">
         <v>3</v>
       </c>
-      <c r="H5" s="295"/>
-      <c r="I5" s="303"/>
+      <c r="H5" s="304"/>
+      <c r="I5" s="298"/>
       <c r="J5" s="12">
         <v>1</v>
       </c>
@@ -7700,16 +7700,16 @@
       <c r="L5" s="12">
         <v>3</v>
       </c>
-      <c r="M5" s="305"/>
-      <c r="N5" s="297"/>
-      <c r="O5" s="301"/>
+      <c r="M5" s="300"/>
+      <c r="N5" s="292"/>
+      <c r="O5" s="296"/>
     </row>
     <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="220" t="str">
         <f>Paėmimas!B6</f>
         <v>XX</v>
       </c>
-      <c r="B6" s="292" t="str">
+      <c r="B6" s="301" t="str">
         <f>Paėmimas!C6</f>
         <v>XXXX</v>
       </c>
@@ -7759,7 +7759,7 @@
     </row>
     <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="34"/>
-      <c r="B7" s="293"/>
+      <c r="B7" s="302"/>
       <c r="C7" s="33">
         <v>2</v>
       </c>
@@ -7796,7 +7796,7 @@
     </row>
     <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="34"/>
-      <c r="B8" s="293"/>
+      <c r="B8" s="302"/>
       <c r="C8" s="33"/>
       <c r="D8" s="89"/>
       <c r="E8" s="176"/>
@@ -7816,7 +7816,7 @@
     </row>
     <row r="9" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A9" s="34"/>
-      <c r="B9" s="293"/>
+      <c r="B9" s="302"/>
       <c r="C9" s="33">
         <v>3</v>
       </c>
@@ -7853,7 +7853,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="34"/>
-      <c r="B10" s="293"/>
+      <c r="B10" s="302"/>
       <c r="C10" s="33"/>
       <c r="D10" s="89"/>
       <c r="E10" s="176"/>
@@ -7870,7 +7870,7 @@
     </row>
     <row r="11" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A11" s="34"/>
-      <c r="B11" s="293"/>
+      <c r="B11" s="302"/>
       <c r="C11" s="33">
         <v>41</v>
       </c>
@@ -7906,7 +7906,7 @@
     </row>
     <row r="12" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="34"/>
-      <c r="B12" s="293"/>
+      <c r="B12" s="302"/>
       <c r="C12" s="112" t="s">
         <v>45</v>
       </c>
@@ -7942,7 +7942,7 @@
     </row>
     <row r="13" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A13" s="34"/>
-      <c r="B13" s="293"/>
+      <c r="B13" s="302"/>
       <c r="C13" s="113" t="s">
         <v>46</v>
       </c>
@@ -7978,7 +7978,7 @@
     </row>
     <row r="14" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A14" s="34"/>
-      <c r="B14" s="293"/>
+      <c r="B14" s="302"/>
       <c r="C14" s="113" t="s">
         <v>47</v>
       </c>
@@ -8014,7 +8014,7 @@
     </row>
     <row r="15" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A15" s="34"/>
-      <c r="B15" s="293"/>
+      <c r="B15" s="302"/>
       <c r="C15" s="114" t="s">
         <v>48</v>
       </c>
@@ -8050,7 +8050,7 @@
     </row>
     <row r="16" spans="1:16" ht="32.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="22"/>
-      <c r="B16" s="294"/>
+      <c r="B16" s="303"/>
       <c r="C16" s="33"/>
       <c r="D16" s="92"/>
       <c r="E16" s="21"/>
@@ -8084,6 +8084,11 @@
     </sortState>
   </autoFilter>
   <mergeCells count="14">
+    <mergeCell ref="B6:B16"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="H4:H5"/>
     <mergeCell ref="J4:L4"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="A2:O2"/>
@@ -8093,11 +8098,6 @@
     <mergeCell ref="O4:O5"/>
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="M4:M5"/>
-    <mergeCell ref="B6:B16"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:H5"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -8173,14 +8173,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8439,21 +8437,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
-    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8478,9 +8475,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Suskaičiuotas lapas H2O ir pusė Aerodinamika su AerodinamikaSK1Funkcija.py
</commit_message>
<xml_diff>
--- a/PVZ1.xlsx
+++ b/PVZ1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agentura2020.sharepoint.com/sites/VidurioLietuvosaplinkostyrimuskyrius/Bendrai naudojami dokumentai/EB7-014 Darbuotojų failai/Tomo/Python 3.14.3/Skaiciavimai/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="156" documentId="8_{6218F508-2438-4EC7-8B4D-5D6F3C7CDB90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CCB77C3-F1CA-4685-9C91-9C1392E2EB9F}"/>
+  <xr:revisionPtr revIDLastSave="157" documentId="8_{6218F508-2438-4EC7-8B4D-5D6F3C7CDB90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B072962-9058-499D-B606-048057C949EB}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="3" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="2" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Compatibility Report" sheetId="4" state="hidden" r:id="rId1"/>
@@ -2695,6 +2695,91 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="29" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -2723,91 +2808,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="29" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="10" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -2818,6 +2818,42 @@
     <xf numFmtId="169" fontId="4" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2833,42 +2869,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -3304,31 +3304,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="D3" s="276" t="s">
+      <c r="D3" s="267" t="s">
         <v>109</v>
       </c>
-      <c r="E3" s="276"/>
-      <c r="F3" s="276"/>
-      <c r="G3" s="276"/>
-      <c r="H3" s="276"/>
-      <c r="I3" s="276"/>
-      <c r="J3" s="276"/>
-      <c r="K3" s="276"/>
-      <c r="L3" s="276"/>
-      <c r="M3" s="276"/>
-      <c r="N3" s="276"/>
-      <c r="O3" s="276"/>
-      <c r="P3" s="276"/>
-      <c r="Q3" s="276"/>
-      <c r="R3" s="276"/>
-      <c r="S3" s="276"/>
-      <c r="T3" s="276"/>
-      <c r="U3" s="276"/>
-      <c r="V3" s="276"/>
-      <c r="W3" s="276"/>
-      <c r="X3" s="276"/>
-      <c r="Y3" s="276"/>
-      <c r="Z3" s="276"/>
+      <c r="E3" s="267"/>
+      <c r="F3" s="267"/>
+      <c r="G3" s="267"/>
+      <c r="H3" s="267"/>
+      <c r="I3" s="267"/>
+      <c r="J3" s="267"/>
+      <c r="K3" s="267"/>
+      <c r="L3" s="267"/>
+      <c r="M3" s="267"/>
+      <c r="N3" s="267"/>
+      <c r="O3" s="267"/>
+      <c r="P3" s="267"/>
+      <c r="Q3" s="267"/>
+      <c r="R3" s="267"/>
+      <c r="S3" s="267"/>
+      <c r="T3" s="267"/>
+      <c r="U3" s="267"/>
+      <c r="V3" s="267"/>
+      <c r="W3" s="267"/>
+      <c r="X3" s="267"/>
+      <c r="Y3" s="267"/>
+      <c r="Z3" s="267"/>
     </row>
     <row r="5" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
@@ -3417,13 +3417,13 @@
       </c>
     </row>
     <row r="6" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="270" t="s">
+      <c r="A6" s="278" t="s">
         <v>148</v>
       </c>
-      <c r="B6" s="277" t="s">
+      <c r="B6" s="268" t="s">
         <v>147</v>
       </c>
-      <c r="C6" s="278" t="s">
+      <c r="C6" s="269" t="s">
         <v>149</v>
       </c>
       <c r="D6" s="135">
@@ -3514,14 +3514,14 @@
         <f>Aerodinamika!G31</f>
         <v>1.2973599999999996</v>
       </c>
-      <c r="AB6" s="273" t="s">
+      <c r="AB6" s="270" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="271"/>
-      <c r="B7" s="277"/>
-      <c r="C7" s="278"/>
+      <c r="A7" s="279"/>
+      <c r="B7" s="268"/>
+      <c r="C7" s="269"/>
       <c r="D7" s="135">
         <v>39</v>
       </c>
@@ -3606,12 +3606,12 @@
         <f>O6*X7</f>
         <v>0.34740732161375365</v>
       </c>
-      <c r="AB7" s="274"/>
+      <c r="AB7" s="271"/>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="271"/>
-      <c r="B8" s="277"/>
-      <c r="C8" s="278"/>
+      <c r="A8" s="279"/>
+      <c r="B8" s="268"/>
+      <c r="C8" s="269"/>
       <c r="D8" s="152">
         <v>71</v>
       </c>
@@ -3662,9 +3662,9 @@
       <c r="S8" s="157"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A9" s="271"/>
-      <c r="B9" s="277"/>
-      <c r="C9" s="278"/>
+      <c r="A9" s="279"/>
+      <c r="B9" s="268"/>
+      <c r="C9" s="269"/>
       <c r="D9" s="135">
         <v>116</v>
       </c>
@@ -3719,9 +3719,9 @@
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A10" s="271"/>
-      <c r="B10" s="277"/>
-      <c r="C10" s="278"/>
+      <c r="A10" s="279"/>
+      <c r="B10" s="268"/>
+      <c r="C10" s="269"/>
       <c r="D10" s="135">
         <v>200</v>
       </c>
@@ -3765,9 +3765,9 @@
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A11" s="271"/>
-      <c r="B11" s="277"/>
-      <c r="C11" s="278"/>
+      <c r="A11" s="279"/>
+      <c r="B11" s="268"/>
+      <c r="C11" s="269"/>
       <c r="D11" s="135">
         <v>284</v>
       </c>
@@ -3811,9 +3811,9 @@
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A12" s="271"/>
-      <c r="B12" s="277"/>
-      <c r="C12" s="278"/>
+      <c r="A12" s="279"/>
+      <c r="B12" s="268"/>
+      <c r="C12" s="269"/>
       <c r="D12" s="135">
         <v>329</v>
       </c>
@@ -3857,9 +3857,9 @@
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A13" s="271"/>
-      <c r="B13" s="277"/>
-      <c r="C13" s="278"/>
+      <c r="A13" s="279"/>
+      <c r="B13" s="268"/>
+      <c r="C13" s="269"/>
       <c r="D13" s="135">
         <v>361</v>
       </c>
@@ -3904,9 +3904,9 @@
       <c r="O13" s="132"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A14" s="271"/>
-      <c r="B14" s="277"/>
-      <c r="C14" s="278"/>
+      <c r="A14" s="279"/>
+      <c r="B14" s="268"/>
+      <c r="C14" s="269"/>
       <c r="D14" s="135">
         <v>388</v>
       </c>
@@ -3954,7 +3954,7 @@
       <c r="U14" s="38"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A15" s="271"/>
+      <c r="A15" s="279"/>
       <c r="B15" s="134"/>
       <c r="C15" s="134"/>
       <c r="D15" s="134"/>
@@ -3976,27 +3976,27 @@
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A16" s="271"/>
+      <c r="A16" s="279"/>
       <c r="B16" s="161"/>
       <c r="C16" s="161"/>
       <c r="D16" s="152" t="s">
         <v>133</v>
       </c>
-      <c r="E16" s="279" t="s">
+      <c r="E16" s="272" t="s">
         <v>134</v>
       </c>
-      <c r="F16" s="280"/>
-      <c r="G16" s="280"/>
-      <c r="H16" s="280"/>
-      <c r="I16" s="280"/>
-      <c r="J16" s="280"/>
-      <c r="K16" s="280"/>
-      <c r="L16" s="280"/>
-      <c r="M16" s="280"/>
-      <c r="N16" s="281"/>
+      <c r="F16" s="273"/>
+      <c r="G16" s="273"/>
+      <c r="H16" s="273"/>
+      <c r="I16" s="273"/>
+      <c r="J16" s="273"/>
+      <c r="K16" s="273"/>
+      <c r="L16" s="273"/>
+      <c r="M16" s="273"/>
+      <c r="N16" s="274"/>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A17" s="271"/>
+      <c r="A17" s="279"/>
       <c r="B17" s="134"/>
       <c r="C17" s="134"/>
       <c r="E17" s="162"/>
@@ -4005,7 +4005,7 @@
       <c r="N17" s="164"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A18" s="271"/>
+      <c r="A18" s="279"/>
       <c r="B18" s="134"/>
       <c r="C18" s="134"/>
       <c r="E18" s="162"/>
@@ -4017,7 +4017,7 @@
       </c>
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A19" s="271"/>
+      <c r="A19" s="279"/>
       <c r="B19" s="134"/>
       <c r="C19" s="134"/>
       <c r="E19" s="38"/>
@@ -4025,37 +4025,37 @@
       <c r="N19" s="164"/>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A20" s="271"/>
+      <c r="A20" s="279"/>
       <c r="B20" s="161"/>
       <c r="C20" s="161"/>
-      <c r="D20" s="275" t="s">
+      <c r="D20" s="281" t="s">
         <v>136</v>
       </c>
-      <c r="E20" s="276"/>
-      <c r="F20" s="276"/>
-      <c r="G20" s="276"/>
-      <c r="H20" s="276"/>
-      <c r="I20" s="276"/>
-      <c r="J20" s="276"/>
-      <c r="K20" s="276"/>
-      <c r="L20" s="276"/>
-      <c r="M20" s="276"/>
-      <c r="N20" s="276"/>
-      <c r="O20" s="276"/>
-      <c r="P20" s="276"/>
-      <c r="Q20" s="276"/>
-      <c r="R20" s="276"/>
-      <c r="S20" s="276"/>
-      <c r="T20" s="276"/>
-      <c r="U20" s="276"/>
-      <c r="V20" s="276"/>
-      <c r="W20" s="276"/>
-      <c r="X20" s="276"/>
-      <c r="Y20" s="276"/>
-      <c r="Z20" s="276"/>
+      <c r="E20" s="267"/>
+      <c r="F20" s="267"/>
+      <c r="G20" s="267"/>
+      <c r="H20" s="267"/>
+      <c r="I20" s="267"/>
+      <c r="J20" s="267"/>
+      <c r="K20" s="267"/>
+      <c r="L20" s="267"/>
+      <c r="M20" s="267"/>
+      <c r="N20" s="267"/>
+      <c r="O20" s="267"/>
+      <c r="P20" s="267"/>
+      <c r="Q20" s="267"/>
+      <c r="R20" s="267"/>
+      <c r="S20" s="267"/>
+      <c r="T20" s="267"/>
+      <c r="U20" s="267"/>
+      <c r="V20" s="267"/>
+      <c r="W20" s="267"/>
+      <c r="X20" s="267"/>
+      <c r="Y20" s="267"/>
+      <c r="Z20" s="267"/>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A21" s="271"/>
+      <c r="A21" s="279"/>
       <c r="B21" s="134"/>
       <c r="C21" s="134"/>
       <c r="D21" s="165"/>
@@ -4072,7 +4072,7 @@
       <c r="O21" s="165"/>
     </row>
     <row r="22" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
-      <c r="A22" s="272"/>
+      <c r="A22" s="280"/>
       <c r="B22" s="9" t="s">
         <v>82</v>
       </c>
@@ -4156,9 +4156,9 @@
       </c>
     </row>
     <row r="23" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="267"/>
-      <c r="B23" s="267"/>
-      <c r="C23" s="267"/>
+      <c r="A23" s="275"/>
+      <c r="B23" s="275"/>
+      <c r="C23" s="275"/>
       <c r="D23" s="135">
         <v>12</v>
       </c>
@@ -4238,12 +4238,12 @@
         <f>Aerodinamika!G31</f>
         <v>1.2973599999999996</v>
       </c>
-      <c r="AB23" s="273"/>
+      <c r="AB23" s="270"/>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A24" s="268"/>
-      <c r="B24" s="268"/>
-      <c r="C24" s="268"/>
+      <c r="A24" s="276"/>
+      <c r="B24" s="276"/>
+      <c r="C24" s="276"/>
       <c r="D24" s="135">
         <v>39</v>
       </c>
@@ -4316,12 +4316,12 @@
         <f>O23*X24</f>
         <v>0.34740732161375365</v>
       </c>
-      <c r="AB24" s="274"/>
+      <c r="AB24" s="271"/>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A25" s="268"/>
-      <c r="B25" s="268"/>
-      <c r="C25" s="268"/>
+      <c r="A25" s="276"/>
+      <c r="B25" s="276"/>
+      <c r="C25" s="276"/>
       <c r="D25" s="152">
         <v>71</v>
       </c>
@@ -4360,9 +4360,9 @@
       <c r="S25" s="157"/>
     </row>
     <row r="26" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A26" s="268"/>
-      <c r="B26" s="268"/>
-      <c r="C26" s="268"/>
+      <c r="A26" s="276"/>
+      <c r="B26" s="276"/>
+      <c r="C26" s="276"/>
       <c r="D26" s="135">
         <v>116</v>
       </c>
@@ -4405,9 +4405,9 @@
       </c>
     </row>
     <row r="27" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A27" s="268"/>
-      <c r="B27" s="268"/>
-      <c r="C27" s="268"/>
+      <c r="A27" s="276"/>
+      <c r="B27" s="276"/>
+      <c r="C27" s="276"/>
       <c r="D27" s="135">
         <v>200</v>
       </c>
@@ -4439,9 +4439,9 @@
       </c>
     </row>
     <row r="28" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A28" s="268"/>
-      <c r="B28" s="268"/>
-      <c r="C28" s="268"/>
+      <c r="A28" s="276"/>
+      <c r="B28" s="276"/>
+      <c r="C28" s="276"/>
       <c r="D28" s="135">
         <v>284</v>
       </c>
@@ -4473,9 +4473,9 @@
       </c>
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A29" s="268"/>
-      <c r="B29" s="268"/>
-      <c r="C29" s="268"/>
+      <c r="A29" s="276"/>
+      <c r="B29" s="276"/>
+      <c r="C29" s="276"/>
       <c r="D29" s="135">
         <v>329</v>
       </c>
@@ -4507,9 +4507,9 @@
       </c>
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A30" s="268"/>
-      <c r="B30" s="268"/>
-      <c r="C30" s="268"/>
+      <c r="A30" s="276"/>
+      <c r="B30" s="276"/>
+      <c r="C30" s="276"/>
       <c r="D30" s="135">
         <v>361</v>
       </c>
@@ -4542,9 +4542,9 @@
       <c r="O30" s="132"/>
     </row>
     <row r="31" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A31" s="269"/>
-      <c r="B31" s="269"/>
-      <c r="C31" s="269"/>
+      <c r="A31" s="277"/>
+      <c r="B31" s="277"/>
+      <c r="C31" s="277"/>
       <c r="D31" s="135">
         <v>388</v>
       </c>
@@ -4582,17 +4582,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="ecyaGde8bRCGGLjxH6/y64hd/Qu1QGpziWOApJzf8uG7KOwveh+XtxYm7qcvHDbOm4wNpJpjwTw6EQ3sZyT0Ww==" saltValue="0y2ywmKlSNb5pUNmtC6Umw==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="11">
-    <mergeCell ref="D3:Z3"/>
-    <mergeCell ref="B6:B14"/>
-    <mergeCell ref="C6:C14"/>
-    <mergeCell ref="AB6:AB7"/>
-    <mergeCell ref="E16:N16"/>
     <mergeCell ref="A23:A31"/>
     <mergeCell ref="B23:B31"/>
     <mergeCell ref="C23:C31"/>
     <mergeCell ref="A6:A22"/>
     <mergeCell ref="AB23:AB24"/>
     <mergeCell ref="D20:Z20"/>
+    <mergeCell ref="D3:Z3"/>
+    <mergeCell ref="B6:B14"/>
+    <mergeCell ref="C6:C14"/>
+    <mergeCell ref="AB6:AB7"/>
+    <mergeCell ref="E16:N16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4638,18 +4638,18 @@
       <c r="I2" s="10"/>
     </row>
     <row r="3" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="260" t="s">
+      <c r="A3" s="282" t="s">
         <v>108</v>
       </c>
-      <c r="B3" s="260"/>
-      <c r="C3" s="260"/>
-      <c r="D3" s="260"/>
-      <c r="E3" s="260"/>
-      <c r="F3" s="260"/>
-      <c r="G3" s="260"/>
-      <c r="H3" s="260"/>
-      <c r="I3" s="260"/>
-      <c r="J3" s="260"/>
+      <c r="B3" s="282"/>
+      <c r="C3" s="282"/>
+      <c r="D3" s="282"/>
+      <c r="E3" s="282"/>
+      <c r="F3" s="282"/>
+      <c r="G3" s="282"/>
+      <c r="H3" s="282"/>
+      <c r="I3" s="282"/>
+      <c r="J3" s="282"/>
     </row>
     <row r="4" spans="1:12" ht="14" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
@@ -4796,46 +4796,46 @@
       <c r="L10" s="46"/>
     </row>
     <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H11" s="261" t="s">
+      <c r="H11" s="283" t="s">
         <v>30</v>
       </c>
-      <c r="I11" s="264" t="s">
+      <c r="I11" s="286" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H12" s="262"/>
-      <c r="I12" s="265"/>
+      <c r="H12" s="284"/>
+      <c r="I12" s="287"/>
     </row>
     <row r="13" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H13" s="262"/>
-      <c r="I13" s="265"/>
+      <c r="H13" s="284"/>
+      <c r="I13" s="287"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H14" s="262"/>
-      <c r="I14" s="265"/>
+      <c r="H14" s="284"/>
+      <c r="I14" s="287"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H15" s="262"/>
-      <c r="I15" s="265"/>
+      <c r="H15" s="284"/>
+      <c r="I15" s="287"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H16" s="262"/>
-      <c r="I16" s="265"/>
+      <c r="H16" s="284"/>
+      <c r="I16" s="287"/>
     </row>
     <row r="17" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H17" s="262"/>
-      <c r="I17" s="265"/>
+      <c r="H17" s="284"/>
+      <c r="I17" s="287"/>
     </row>
     <row r="18" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H18" s="263"/>
-      <c r="I18" s="265"/>
+      <c r="H18" s="285"/>
+      <c r="I18" s="287"/>
     </row>
     <row r="19" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I19" s="265"/>
+      <c r="I19" s="287"/>
     </row>
     <row r="20" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I20" s="266"/>
+      <c r="I20" s="288"/>
     </row>
     <row r="21" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I21" s="57"/>
@@ -4854,7 +4854,7 @@
       <c r="I26" s="56"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="vsA/nwLr0Dhf9eh67ecTlH1FUVwPEXu619v7Knny3aw2Q7fxwLaiHXjlaMzDBn74tTq+iJFURX0oZc6EcWh/fA==" saltValue="G3/kUvf5HPy2Ci9qKPTF0g==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="3">
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="H11:H18"/>
@@ -4900,35 +4900,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="287" t="s">
+      <c r="C1" s="265" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="287"/>
+      <c r="D1" s="265"/>
       <c r="E1" s="15"/>
       <c r="S1" s="16"/>
     </row>
     <row r="2" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="288" t="s">
+      <c r="A2" s="266" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="288"/>
-      <c r="C2" s="288"/>
-      <c r="D2" s="288"/>
-      <c r="E2" s="288"/>
-      <c r="F2" s="288"/>
-      <c r="G2" s="288"/>
-      <c r="H2" s="288"/>
-      <c r="I2" s="288"/>
-      <c r="J2" s="288"/>
-      <c r="K2" s="288"/>
-      <c r="L2" s="288"/>
-      <c r="M2" s="288"/>
-      <c r="N2" s="288"/>
-      <c r="O2" s="288"/>
-      <c r="P2" s="288"/>
-      <c r="Q2" s="288"/>
-      <c r="R2" s="288"/>
-      <c r="S2" s="288"/>
+      <c r="B2" s="266"/>
+      <c r="C2" s="266"/>
+      <c r="D2" s="266"/>
+      <c r="E2" s="266"/>
+      <c r="F2" s="266"/>
+      <c r="G2" s="266"/>
+      <c r="H2" s="266"/>
+      <c r="I2" s="266"/>
+      <c r="J2" s="266"/>
+      <c r="K2" s="266"/>
+      <c r="L2" s="266"/>
+      <c r="M2" s="266"/>
+      <c r="N2" s="266"/>
+      <c r="O2" s="266"/>
+      <c r="P2" s="266"/>
+      <c r="Q2" s="266"/>
+      <c r="R2" s="266"/>
+      <c r="S2" s="266"/>
     </row>
     <row r="3" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
@@ -5036,7 +5036,7 @@
       <c r="B6" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="C6" s="283" t="str">
+      <c r="C6" s="261" t="str">
         <f>Greitis!C6</f>
         <v>XXXX</v>
       </c>
@@ -5116,7 +5116,7 @@
     <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" s="37"/>
       <c r="B7" s="34"/>
-      <c r="C7" s="284"/>
+      <c r="C7" s="262"/>
       <c r="D7" s="19"/>
       <c r="E7" s="20"/>
       <c r="F7" s="185">
@@ -5187,7 +5187,7 @@
     <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8" s="37"/>
       <c r="B8" s="34"/>
-      <c r="C8" s="284"/>
+      <c r="C8" s="262"/>
       <c r="D8" s="19"/>
       <c r="E8" s="20"/>
       <c r="F8" s="185">
@@ -5258,7 +5258,7 @@
     <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9" s="49"/>
       <c r="B9" s="49"/>
-      <c r="C9" s="284"/>
+      <c r="C9" s="262"/>
       <c r="D9" s="49"/>
       <c r="E9" s="49"/>
       <c r="F9" s="185">
@@ -5332,7 +5332,7 @@
     <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="49"/>
       <c r="B10" s="49"/>
-      <c r="C10" s="284"/>
+      <c r="C10" s="262"/>
       <c r="D10" s="49"/>
       <c r="E10" s="49"/>
       <c r="F10" s="185">
@@ -5382,13 +5382,13 @@
       </c>
       <c r="R10" s="49"/>
       <c r="S10" s="49"/>
-      <c r="T10" s="286" t="s">
+      <c r="T10" s="264" t="s">
         <v>32</v>
       </c>
-      <c r="U10" s="286" t="s">
+      <c r="U10" s="264" t="s">
         <v>33</v>
       </c>
-      <c r="V10" s="282" t="s">
+      <c r="V10" s="260" t="s">
         <v>40</v>
       </c>
       <c r="X10" s="240">
@@ -5403,7 +5403,7 @@
     <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11" s="49"/>
       <c r="B11" s="49"/>
-      <c r="C11" s="284"/>
+      <c r="C11" s="262"/>
       <c r="D11" s="49"/>
       <c r="E11" s="49"/>
       <c r="F11" s="185">
@@ -5453,9 +5453,9 @@
       </c>
       <c r="R11" s="49"/>
       <c r="S11" s="49"/>
-      <c r="T11" s="286"/>
-      <c r="U11" s="286"/>
-      <c r="V11" s="282"/>
+      <c r="T11" s="264"/>
+      <c r="U11" s="264"/>
+      <c r="V11" s="260"/>
       <c r="X11" s="240">
         <f>Greitis!E11</f>
         <v>0.14000000000000001</v>
@@ -5468,7 +5468,7 @@
     <row r="12" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="49"/>
       <c r="B12" s="49"/>
-      <c r="C12" s="284"/>
+      <c r="C12" s="262"/>
       <c r="D12" s="49"/>
       <c r="E12" s="49"/>
       <c r="F12" s="185">
@@ -5518,9 +5518,9 @@
       </c>
       <c r="R12" s="49"/>
       <c r="S12" s="49"/>
-      <c r="T12" s="286"/>
-      <c r="U12" s="286"/>
-      <c r="V12" s="282"/>
+      <c r="T12" s="264"/>
+      <c r="U12" s="264"/>
+      <c r="V12" s="260"/>
       <c r="X12" s="240">
         <f>Greitis!E12</f>
         <v>0.14000000000000001</v>
@@ -5533,7 +5533,7 @@
     <row r="13" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="49"/>
       <c r="B13" s="49"/>
-      <c r="C13" s="284"/>
+      <c r="C13" s="262"/>
       <c r="D13" s="49"/>
       <c r="E13" s="49"/>
       <c r="F13" s="185">
@@ -5595,7 +5595,7 @@
     <row r="14" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="36"/>
       <c r="B14" s="36"/>
-      <c r="C14" s="285"/>
+      <c r="C14" s="263"/>
       <c r="D14" s="36"/>
       <c r="E14" s="36"/>
       <c r="F14" s="185">
@@ -5693,7 +5693,7 @@
         <f t="shared" si="27"/>
         <v>XX</v>
       </c>
-      <c r="C19" s="283" t="str">
+      <c r="C19" s="261" t="str">
         <f t="shared" si="27"/>
         <v>XXXX</v>
       </c>
@@ -5769,7 +5769,7 @@
     <row r="20" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A20" s="37"/>
       <c r="B20" s="34"/>
-      <c r="C20" s="284"/>
+      <c r="C20" s="262"/>
       <c r="D20" s="19"/>
       <c r="E20" s="20"/>
       <c r="F20" s="185">
@@ -5831,7 +5831,7 @@
     <row r="21" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A21" s="37"/>
       <c r="B21" s="34"/>
-      <c r="C21" s="284"/>
+      <c r="C21" s="262"/>
       <c r="D21" s="19"/>
       <c r="E21" s="20"/>
       <c r="F21" s="185">
@@ -5893,7 +5893,7 @@
     <row r="22" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A22" s="49"/>
       <c r="B22" s="49"/>
-      <c r="C22" s="284"/>
+      <c r="C22" s="262"/>
       <c r="D22" s="49"/>
       <c r="E22" s="49"/>
       <c r="F22" s="185">
@@ -5955,7 +5955,7 @@
     <row r="23" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A23" s="49"/>
       <c r="B23" s="49"/>
-      <c r="C23" s="284"/>
+      <c r="C23" s="262"/>
       <c r="D23" s="49"/>
       <c r="E23" s="49"/>
       <c r="F23" s="185">
@@ -6017,7 +6017,7 @@
     <row r="24" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A24" s="49"/>
       <c r="B24" s="49"/>
-      <c r="C24" s="284"/>
+      <c r="C24" s="262"/>
       <c r="D24" s="49"/>
       <c r="E24" s="49"/>
       <c r="F24" s="185">
@@ -6079,7 +6079,7 @@
     <row r="25" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A25" s="49"/>
       <c r="B25" s="49"/>
-      <c r="C25" s="284"/>
+      <c r="C25" s="262"/>
       <c r="D25" s="49"/>
       <c r="E25" s="49"/>
       <c r="F25" s="185">
@@ -6141,7 +6141,7 @@
     <row r="26" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A26" s="49"/>
       <c r="B26" s="49"/>
-      <c r="C26" s="284"/>
+      <c r="C26" s="262"/>
       <c r="D26" s="49"/>
       <c r="E26" s="49"/>
       <c r="F26" s="185">
@@ -6203,7 +6203,7 @@
     <row r="27" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A27" s="36"/>
       <c r="B27" s="36"/>
-      <c r="C27" s="285"/>
+      <c r="C27" s="263"/>
       <c r="D27" s="36"/>
       <c r="E27" s="36"/>
       <c r="F27" s="185">
@@ -6383,10 +6383,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="287" t="s">
+      <c r="C1" s="265" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="287"/>
+      <c r="D1" s="265"/>
       <c r="Q1" s="16"/>
     </row>
     <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -6464,7 +6464,7 @@
         <f>Paėmimas!B6</f>
         <v>XX</v>
       </c>
-      <c r="C6" s="283" t="str">
+      <c r="C6" s="261" t="str">
         <f>Paėmimas!C6</f>
         <v>XXXX</v>
       </c>
@@ -6516,7 +6516,7 @@
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="59"/>
       <c r="B7" s="23"/>
-      <c r="C7" s="284"/>
+      <c r="C7" s="262"/>
       <c r="D7" s="193">
         <f>Paėmimas!L7</f>
         <v>0.05</v>
@@ -6553,7 +6553,7 @@
     <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="59"/>
       <c r="B8" s="23"/>
-      <c r="C8" s="284"/>
+      <c r="C8" s="262"/>
       <c r="D8" s="193">
         <f>Paėmimas!L8</f>
         <v>0.05</v>
@@ -6590,7 +6590,7 @@
     <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="59"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="284"/>
+      <c r="C9" s="262"/>
       <c r="D9" s="193">
         <f>Paėmimas!L9</f>
         <v>0.05</v>
@@ -6627,7 +6627,7 @@
     <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="59"/>
       <c r="B10" s="23"/>
-      <c r="C10" s="284"/>
+      <c r="C10" s="262"/>
       <c r="D10" s="193">
         <f>Paėmimas!L10</f>
         <v>0.05</v>
@@ -6664,7 +6664,7 @@
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="59"/>
       <c r="B11" s="23"/>
-      <c r="C11" s="284"/>
+      <c r="C11" s="262"/>
       <c r="D11" s="193">
         <f>Paėmimas!L11</f>
         <v>0.05</v>
@@ -6701,7 +6701,7 @@
     <row r="12" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="59"/>
       <c r="B12" s="23"/>
-      <c r="C12" s="284"/>
+      <c r="C12" s="262"/>
       <c r="D12" s="193">
         <f>Paėmimas!L12</f>
         <v>0.05</v>
@@ -6738,7 +6738,7 @@
     <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="59"/>
       <c r="B13" s="23"/>
-      <c r="C13" s="284"/>
+      <c r="C13" s="262"/>
       <c r="D13" s="193">
         <f>Paėmimas!L13</f>
         <v>0.05</v>
@@ -6775,7 +6775,7 @@
     <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="61"/>
       <c r="B14" s="62"/>
-      <c r="C14" s="285"/>
+      <c r="C14" s="263"/>
       <c r="D14" s="193">
         <f>Paėmimas!L14</f>
         <v>0.05</v>
@@ -6858,7 +6858,7 @@
         <f>Paėmimas!B19</f>
         <v>XX</v>
       </c>
-      <c r="C19" s="283" t="str">
+      <c r="C19" s="261" t="str">
         <f>Paėmimas!C19</f>
         <v>XXXX</v>
       </c>
@@ -6910,7 +6910,7 @@
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="59"/>
       <c r="B20" s="23"/>
-      <c r="C20" s="284"/>
+      <c r="C20" s="262"/>
       <c r="D20" s="193">
         <f>Paėmimas!L20</f>
         <v>0.05</v>
@@ -6947,7 +6947,7 @@
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="59"/>
       <c r="B21" s="23"/>
-      <c r="C21" s="284"/>
+      <c r="C21" s="262"/>
       <c r="D21" s="193">
         <f>Paėmimas!L21</f>
         <v>0.05</v>
@@ -6984,7 +6984,7 @@
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="59"/>
       <c r="B22" s="23"/>
-      <c r="C22" s="284"/>
+      <c r="C22" s="262"/>
       <c r="D22" s="193">
         <f>Paėmimas!L22</f>
         <v>0.05</v>
@@ -7021,7 +7021,7 @@
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="59"/>
       <c r="B23" s="23"/>
-      <c r="C23" s="284"/>
+      <c r="C23" s="262"/>
       <c r="D23" s="193">
         <f>Paėmimas!L23</f>
         <v>0.05</v>
@@ -7058,7 +7058,7 @@
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="59"/>
       <c r="B24" s="23"/>
-      <c r="C24" s="284"/>
+      <c r="C24" s="262"/>
       <c r="D24" s="193">
         <f>Paėmimas!L24</f>
         <v>0.05</v>
@@ -7095,7 +7095,7 @@
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="59"/>
       <c r="B25" s="23"/>
-      <c r="C25" s="284"/>
+      <c r="C25" s="262"/>
       <c r="D25" s="193">
         <f>Paėmimas!L25</f>
         <v>0.05</v>
@@ -7132,7 +7132,7 @@
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="59"/>
       <c r="B26" s="23"/>
-      <c r="C26" s="284"/>
+      <c r="C26" s="262"/>
       <c r="D26" s="193">
         <f>Paėmimas!L26</f>
         <v>0.05</v>
@@ -7169,7 +7169,7 @@
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="61"/>
       <c r="B27" s="62"/>
-      <c r="C27" s="285"/>
+      <c r="C27" s="263"/>
       <c r="D27" s="193">
         <f>Paėmimas!L27</f>
         <v>0.05</v>
@@ -7364,10 +7364,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="287" t="s">
+      <c r="C1" s="265" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="287"/>
+      <c r="D1" s="265"/>
       <c r="R1" s="16"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -7620,12 +7620,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="287" t="s">
+      <c r="C1" s="265" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="287"/>
-      <c r="E1" s="287"/>
-      <c r="F1" s="287"/>
+      <c r="D1" s="265"/>
+      <c r="E1" s="265"/>
+      <c r="F1" s="265"/>
     </row>
     <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="289" t="s">
@@ -7647,49 +7647,49 @@
       <c r="O2" s="289"/>
     </row>
     <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="298" t="s">
+      <c r="A4" s="293" t="s">
         <v>82</v>
       </c>
-      <c r="B4" s="298" t="s">
+      <c r="B4" s="293" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="295" t="s">
+      <c r="C4" s="304" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="295" t="s">
+      <c r="D4" s="304" t="s">
         <v>84</v>
       </c>
-      <c r="E4" s="295" t="s">
+      <c r="E4" s="304" t="s">
         <v>85</v>
       </c>
-      <c r="F4" s="295"/>
-      <c r="G4" s="295"/>
-      <c r="H4" s="295" t="s">
+      <c r="F4" s="304"/>
+      <c r="G4" s="304"/>
+      <c r="H4" s="304" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="302" t="s">
+      <c r="I4" s="297" t="s">
         <v>86</v>
       </c>
-      <c r="J4" s="297" t="s">
+      <c r="J4" s="292" t="s">
         <v>87</v>
       </c>
-      <c r="K4" s="297"/>
-      <c r="L4" s="297"/>
-      <c r="M4" s="304" t="s">
+      <c r="K4" s="292"/>
+      <c r="L4" s="292"/>
+      <c r="M4" s="299" t="s">
         <v>88</v>
       </c>
-      <c r="N4" s="297" t="s">
+      <c r="N4" s="292" t="s">
         <v>15</v>
       </c>
-      <c r="O4" s="300" t="s">
+      <c r="O4" s="295" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="299"/>
-      <c r="B5" s="299"/>
-      <c r="C5" s="296"/>
-      <c r="D5" s="295"/>
+      <c r="A5" s="294"/>
+      <c r="B5" s="294"/>
+      <c r="C5" s="305"/>
+      <c r="D5" s="304"/>
       <c r="E5" s="116">
         <v>1</v>
       </c>
@@ -7699,8 +7699,8 @@
       <c r="G5" s="116">
         <v>3</v>
       </c>
-      <c r="H5" s="295"/>
-      <c r="I5" s="303"/>
+      <c r="H5" s="304"/>
+      <c r="I5" s="298"/>
       <c r="J5" s="12">
         <v>1</v>
       </c>
@@ -7710,16 +7710,16 @@
       <c r="L5" s="12">
         <v>3</v>
       </c>
-      <c r="M5" s="305"/>
-      <c r="N5" s="297"/>
-      <c r="O5" s="301"/>
+      <c r="M5" s="300"/>
+      <c r="N5" s="292"/>
+      <c r="O5" s="296"/>
     </row>
     <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="220" t="str">
         <f>Paėmimas!B6</f>
         <v>XX</v>
       </c>
-      <c r="B6" s="292" t="str">
+      <c r="B6" s="301" t="str">
         <f>Paėmimas!C6</f>
         <v>XXXX</v>
       </c>
@@ -7769,7 +7769,7 @@
     </row>
     <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="34"/>
-      <c r="B7" s="293"/>
+      <c r="B7" s="302"/>
       <c r="C7" s="33">
         <v>2</v>
       </c>
@@ -7806,7 +7806,7 @@
     </row>
     <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="34"/>
-      <c r="B8" s="293"/>
+      <c r="B8" s="302"/>
       <c r="C8" s="33"/>
       <c r="D8" s="89"/>
       <c r="E8" s="176"/>
@@ -7826,7 +7826,7 @@
     </row>
     <row r="9" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A9" s="34"/>
-      <c r="B9" s="293"/>
+      <c r="B9" s="302"/>
       <c r="C9" s="33">
         <v>3</v>
       </c>
@@ -7863,7 +7863,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="34"/>
-      <c r="B10" s="293"/>
+      <c r="B10" s="302"/>
       <c r="C10" s="33"/>
       <c r="D10" s="89"/>
       <c r="E10" s="176"/>
@@ -7880,7 +7880,7 @@
     </row>
     <row r="11" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A11" s="34"/>
-      <c r="B11" s="293"/>
+      <c r="B11" s="302"/>
       <c r="C11" s="33">
         <v>41</v>
       </c>
@@ -7916,7 +7916,7 @@
     </row>
     <row r="12" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="34"/>
-      <c r="B12" s="293"/>
+      <c r="B12" s="302"/>
       <c r="C12" s="112" t="s">
         <v>45</v>
       </c>
@@ -7952,7 +7952,7 @@
     </row>
     <row r="13" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A13" s="34"/>
-      <c r="B13" s="293"/>
+      <c r="B13" s="302"/>
       <c r="C13" s="113" t="s">
         <v>46</v>
       </c>
@@ -7988,7 +7988,7 @@
     </row>
     <row r="14" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A14" s="34"/>
-      <c r="B14" s="293"/>
+      <c r="B14" s="302"/>
       <c r="C14" s="113" t="s">
         <v>47</v>
       </c>
@@ -8024,7 +8024,7 @@
     </row>
     <row r="15" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A15" s="34"/>
-      <c r="B15" s="293"/>
+      <c r="B15" s="302"/>
       <c r="C15" s="114" t="s">
         <v>48</v>
       </c>
@@ -8060,7 +8060,7 @@
     </row>
     <row r="16" spans="1:16" ht="32.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="22"/>
-      <c r="B16" s="294"/>
+      <c r="B16" s="303"/>
       <c r="C16" s="33"/>
       <c r="D16" s="92"/>
       <c r="E16" s="21"/>
@@ -8094,6 +8094,11 @@
     </sortState>
   </autoFilter>
   <mergeCells count="14">
+    <mergeCell ref="B6:B16"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="H4:H5"/>
     <mergeCell ref="J4:L4"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="A2:O2"/>
@@ -8103,11 +8108,6 @@
     <mergeCell ref="O4:O5"/>
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="M4:M5"/>
-    <mergeCell ref="B6:B16"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:H5"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -8183,6 +8183,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentas" ma:contentTypeID="0x010100BAB57CF81AE55C4698AAD22D302297F0" ma:contentTypeVersion="18" ma:contentTypeDescription="Kurkite naują dokumentą." ma:contentTypeScope="" ma:versionID="49ab401eb4052690d2a2629974c22fd6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="453e7e53-5eb2-45cf-b2ab-34c867e554b8" xmlns:ns3="aa0d983d-359a-438c-9953-3af1a8ac0831" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ab9969d50e0b13c63bc5bd0499c928dc" ns2:_="" ns3:_="">
     <xsd:import namespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
@@ -8437,27 +8457,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0108C608-980F-44FC-9F17-65C384873DE6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8474,23 +8493,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
-    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>